<commit_message>
Bump Python to 3.14 and switch default decimator
Update CI and release workflows to use Python 3.14 and adjust docs/comments (README, requirements.txt). Rename default pipeline from "QEM" to "DecimatePro" (evaluation/experiment_runtime.py, runtime files) and update measured evaluation data (CSV/JSON files and evaluation_tracker.xlsx) to reflect new decimator and benchmark results.
</commit_message>
<xml_diff>
--- a/evaluation/evaluation_tracker.xlsx
+++ b/evaluation/evaluation_tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnniDin00\Documents\GitHub\adaptive-remesher\evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62230777-2A3B-4E63-A432-E5CA5FDF69A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C80CE13C-11F8-4713-961A-EF29D8D5BD72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="236">
   <si>
     <t>Adaptive Remesher — Evaluation Data Tracker</t>
   </si>
@@ -450,7 +450,7 @@
     <t>Does bidirectional error-guided protection reduce geometric error, at the cost of additional protected geometry and reduced simplification?</t>
   </si>
   <si>
-    <t>Error threshold tau (E_max) used for the 'Above threshold' column below:</t>
+    <t>Error threshold tau, as a FRACTION of each model's bounding-box diagonal (as in the app: 0.01 = 1%), used for the 'Above threshold' column below:</t>
   </si>
   <si>
     <t>Config (No refinement / Bidirectional refinement)</t>
@@ -483,6 +483,12 @@
     <t>Above threshold?</t>
   </si>
   <si>
+    <t>Bbox diagonal</t>
+  </si>
+  <si>
+    <t>E_max pooled (% of diagonal)</t>
+  </si>
+  <si>
     <t>No refinement</t>
   </si>
   <si>
@@ -744,17 +750,18 @@
     <t>T_Other (s)</t>
   </si>
   <si>
-    <t>Default pipeline (QEM, 90%, UV+auto-error protection)</t>
+    <t>Default pipeline (DecimatePro, 90%, UV+auto-error protection)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -809,6 +816,11 @@
       <color rgb="FF808080"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -860,7 +872,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -889,6 +901,9 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
@@ -1369,12 +1384,12 @@
   <sheetData>
     <row r="1" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1385,28 +1400,28 @@
         <v>109</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>39</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>40</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -1414,7 +1429,7 @@
         <v>45</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C5" s="7">
         <v>59996</v>
@@ -1447,7 +1462,7 @@
         <v>45</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C6" s="7">
         <v>20228</v>
@@ -1480,7 +1495,7 @@
         <v>52</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C7" s="7">
         <v>15000</v>
@@ -1513,7 +1528,7 @@
         <v>52</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C8" s="7">
         <v>6312</v>
@@ -1546,7 +1561,7 @@
         <v>55</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C9" s="7">
         <v>130504</v>
@@ -1579,7 +1594,7 @@
         <v>55</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C10" s="7">
         <v>36140</v>
@@ -1612,7 +1627,7 @@
         <v>58</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C11" s="7">
         <v>1473</v>
@@ -1645,7 +1660,7 @@
         <v>58</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C12" s="7">
         <v>1386</v>
@@ -1678,7 +1693,7 @@
         <v>62</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C13" s="7">
         <v>13790</v>
@@ -1711,7 +1726,7 @@
         <v>62</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C14" s="7">
         <v>11708</v>
@@ -1744,7 +1759,7 @@
         <v>64</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C15" s="7">
         <v>2752</v>
@@ -1777,7 +1792,7 @@
         <v>64</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C16" s="7">
         <v>2036</v>
@@ -1810,7 +1825,7 @@
         <v>66</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C17" s="7">
         <v>3410</v>
@@ -1843,7 +1858,7 @@
         <v>66</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C18" s="7">
         <v>3192</v>
@@ -1876,7 +1891,7 @@
         <v>69</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C19" s="7">
         <v>2926</v>
@@ -1909,7 +1924,7 @@
         <v>69</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C20" s="7">
         <v>2642</v>
@@ -1942,7 +1957,7 @@
         <v>71</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C21" s="7">
         <v>211874</v>
@@ -1975,7 +1990,7 @@
         <v>71</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C22" s="7">
         <v>52160</v>
@@ -2008,7 +2023,7 @@
         <v>75</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C23" s="7">
         <v>446670</v>
@@ -2041,7 +2056,7 @@
         <v>75</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C24" s="7">
         <v>138308</v>
@@ -2074,7 +2089,7 @@
         <v>78</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C25" s="7">
         <v>108958</v>
@@ -2107,7 +2122,7 @@
         <v>78</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C26" s="7">
         <v>21364</v>
@@ -2140,7 +2155,7 @@
         <v>80</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C27" s="7">
         <v>405680</v>
@@ -2173,7 +2188,7 @@
         <v>80</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C28" s="7">
         <v>251322</v>
@@ -2206,7 +2221,7 @@
         <v>83</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C29" s="7">
         <v>5912</v>
@@ -2239,7 +2254,7 @@
         <v>83</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C30" s="7">
         <v>3270</v>
@@ -2272,7 +2287,7 @@
         <v>88</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C31" s="7">
         <v>16694</v>
@@ -2305,7 +2320,7 @@
         <v>88</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C32" s="7">
         <v>13858</v>
@@ -2338,7 +2353,7 @@
         <v>90</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C33" s="7">
         <v>63998</v>
@@ -2371,7 +2386,7 @@
         <v>90</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C34" s="7">
         <v>23366</v>
@@ -2404,7 +2419,7 @@
         <v>93</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C35" s="7">
         <v>69451</v>
@@ -2437,7 +2452,7 @@
         <v>93</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C36" s="7">
         <v>8112</v>
@@ -2470,7 +2485,7 @@
         <v>97</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C37" s="7">
         <v>345944</v>
@@ -2503,7 +2518,7 @@
         <v>97</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C38" s="7">
         <v>48760</v>
@@ -2536,7 +2551,7 @@
         <v>99</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C39" s="7">
         <v>1869988</v>
@@ -2569,7 +2584,7 @@
         <v>99</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C40" s="7">
         <v>186994</v>
@@ -2602,7 +2617,7 @@
         <v>104</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C41" s="7">
         <v>31400</v>
@@ -2635,7 +2650,7 @@
         <v>104</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C42" s="7">
         <v>21252</v>
@@ -2684,12 +2699,12 @@
   <sheetData>
     <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2703,19 +2718,19 @@
         <v>109</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -2726,19 +2741,19 @@
         <v>59996</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D5" s="7">
-        <v>0.443</v>
+        <v>0.45650000000000002</v>
       </c>
       <c r="E5" s="7">
-        <v>0.16689999999999999</v>
+        <v>0.19420000000000001</v>
       </c>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
       <c r="H5" s="15">
         <f t="shared" ref="H5:H29" si="0">IFERROR(D5-SUM(E5:G5),"")</f>
-        <v>0.27610000000000001</v>
+        <v>0.26229999999999998</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -2749,19 +2764,19 @@
         <v>15000</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D6" s="7">
-        <v>0.1736</v>
+        <v>0.1956</v>
       </c>
       <c r="E6" s="7">
-        <v>3.5499999999999997E-2</v>
+        <v>4.7E-2</v>
       </c>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
       <c r="H6" s="15">
         <f t="shared" si="0"/>
-        <v>0.1381</v>
+        <v>0.14860000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -2772,19 +2787,19 @@
         <v>130504</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D7" s="7">
-        <v>0.90249999999999997</v>
+        <v>0.92090000000000005</v>
       </c>
       <c r="E7" s="7">
-        <v>0.35870000000000002</v>
+        <v>0.38979999999999998</v>
       </c>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
       <c r="H7" s="15">
         <f t="shared" si="0"/>
-        <v>0.54379999999999995</v>
+        <v>0.53110000000000013</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -2795,19 +2810,19 @@
         <v>1473</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D8" s="7">
-        <v>1.43E-2</v>
+        <v>1.9400000000000001E-2</v>
       </c>
       <c r="E8" s="7">
-        <v>5.5999999999999999E-3</v>
+        <v>9.9000000000000008E-3</v>
       </c>
       <c r="F8" s="7"/>
       <c r="G8" s="7"/>
       <c r="H8" s="15">
         <f t="shared" si="0"/>
-        <v>8.6999999999999994E-3</v>
+        <v>9.4999999999999998E-3</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -2818,19 +2833,19 @@
         <v>13790</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D9" s="7">
-        <v>0.2366</v>
+        <v>0.2646</v>
       </c>
       <c r="E9" s="7">
-        <v>2.2800000000000001E-2</v>
+        <v>3.7400000000000003E-2</v>
       </c>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
       <c r="H9" s="15">
         <f t="shared" si="0"/>
-        <v>0.21379999999999999</v>
+        <v>0.22720000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -2841,19 +2856,19 @@
         <v>2752</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D10" s="7">
-        <v>4.1599999999999998E-2</v>
+        <v>5.3800000000000001E-2</v>
       </c>
       <c r="E10" s="7">
-        <v>7.9000000000000008E-3</v>
+        <v>1.43E-2</v>
       </c>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
       <c r="H10" s="15">
         <f t="shared" si="0"/>
-        <v>3.3699999999999994E-2</v>
+        <v>3.95E-2</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -2864,19 +2879,19 @@
         <v>3410</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D11" s="7">
-        <v>3.1300000000000001E-2</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="E11" s="7">
-        <v>1.14E-2</v>
+        <v>1.9800000000000002E-2</v>
       </c>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
       <c r="H11" s="15">
         <f t="shared" si="0"/>
-        <v>1.9900000000000001E-2</v>
+        <v>2.12E-2</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -2887,19 +2902,19 @@
         <v>2926</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D12" s="7">
-        <v>7.6799999999999993E-2</v>
+        <v>9.3600000000000003E-2</v>
       </c>
       <c r="E12" s="7">
-        <v>1.0500000000000001E-2</v>
+        <v>1.6400000000000001E-2</v>
       </c>
       <c r="F12" s="7"/>
       <c r="G12" s="7"/>
       <c r="H12" s="15">
         <f t="shared" si="0"/>
-        <v>6.6299999999999998E-2</v>
+        <v>7.7200000000000005E-2</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -2910,19 +2925,19 @@
         <v>211874</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D13" s="7">
-        <v>1.5871999999999999</v>
+        <v>1.5322</v>
       </c>
       <c r="E13" s="7">
-        <v>0.73780000000000001</v>
+        <v>0.72789999999999999</v>
       </c>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
       <c r="H13" s="15">
         <f t="shared" si="0"/>
-        <v>0.84939999999999993</v>
+        <v>0.80430000000000001</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -2933,19 +2948,19 @@
         <v>446670</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D14" s="7">
-        <v>3.5674999999999999</v>
+        <v>3.7456</v>
       </c>
       <c r="E14" s="7">
-        <v>1.5348999999999999</v>
+        <v>1.7293000000000001</v>
       </c>
       <c r="F14" s="7"/>
       <c r="G14" s="7"/>
       <c r="H14" s="15">
         <f t="shared" si="0"/>
-        <v>2.0326</v>
+        <v>2.0163000000000002</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -2956,19 +2971,19 @@
         <v>108958</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D15" s="7">
-        <v>0.91069999999999995</v>
+        <v>0.91800000000000004</v>
       </c>
       <c r="E15" s="7">
-        <v>0.34150000000000003</v>
+        <v>0.36420000000000002</v>
       </c>
       <c r="F15" s="7"/>
       <c r="G15" s="7"/>
       <c r="H15" s="15">
         <f t="shared" si="0"/>
-        <v>0.56919999999999993</v>
+        <v>0.55380000000000007</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -2979,19 +2994,19 @@
         <v>405680</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D16" s="7">
-        <v>4.1795</v>
+        <v>4.5187999999999997</v>
       </c>
       <c r="E16" s="7">
-        <v>0.91300000000000003</v>
+        <v>1.1801999999999999</v>
       </c>
       <c r="F16" s="7"/>
       <c r="G16" s="7"/>
       <c r="H16" s="15">
         <f t="shared" si="0"/>
-        <v>3.2664999999999997</v>
+        <v>3.3385999999999996</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -3002,19 +3017,19 @@
         <v>5912</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D17" s="7">
-        <v>5.7700000000000001E-2</v>
+        <v>0.12820000000000001</v>
       </c>
       <c r="E17" s="7">
-        <v>1.3599999999999999E-2</v>
+        <v>2.9700000000000001E-2</v>
       </c>
       <c r="F17" s="7"/>
       <c r="G17" s="7"/>
       <c r="H17" s="15">
         <f t="shared" si="0"/>
-        <v>4.41E-2</v>
+        <v>9.8500000000000004E-2</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -3025,19 +3040,19 @@
         <v>16694</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D18" s="7">
-        <v>0.16619999999999999</v>
+        <v>0.18909999999999999</v>
       </c>
       <c r="E18" s="7">
-        <v>3.15E-2</v>
+        <v>5.8500000000000003E-2</v>
       </c>
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
       <c r="H18" s="15">
         <f t="shared" si="0"/>
-        <v>0.13469999999999999</v>
+        <v>0.13059999999999999</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -3048,19 +3063,19 @@
         <v>63998</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D19" s="7">
-        <v>0.41959999999999997</v>
+        <v>0.46</v>
       </c>
       <c r="E19" s="7">
-        <v>0.1583</v>
+        <v>0.19950000000000001</v>
       </c>
       <c r="F19" s="7"/>
       <c r="G19" s="7"/>
       <c r="H19" s="15">
         <f t="shared" si="0"/>
-        <v>0.26129999999999998</v>
+        <v>0.26050000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -3071,19 +3086,19 @@
         <v>69451</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D20" s="7">
-        <v>1.091</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="E20" s="7">
-        <v>0.19409999999999999</v>
+        <v>0.19270000000000001</v>
       </c>
       <c r="F20" s="7"/>
       <c r="G20" s="7"/>
       <c r="H20" s="15">
         <f t="shared" si="0"/>
-        <v>0.89690000000000003</v>
+        <v>0.91730000000000012</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -3094,19 +3109,19 @@
         <v>345944</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D21" s="7">
-        <v>3.0106999999999999</v>
+        <v>2.7427999999999999</v>
       </c>
       <c r="E21" s="7">
-        <v>1.7212000000000001</v>
+        <v>1.5616000000000001</v>
       </c>
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
       <c r="H21" s="15">
         <f t="shared" si="0"/>
-        <v>1.2894999999999999</v>
+        <v>1.1811999999999998</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -3117,19 +3132,19 @@
         <v>1869988</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D22" s="7">
-        <v>30.728400000000001</v>
+        <v>33.584800000000001</v>
       </c>
       <c r="E22" s="7">
-        <v>0.90859999999999996</v>
+        <v>12.879300000000001</v>
       </c>
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
       <c r="H22" s="15">
         <f t="shared" si="0"/>
-        <v>29.819800000000001</v>
+        <v>20.705500000000001</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -3140,19 +3155,19 @@
         <v>31400</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D23" s="7">
-        <v>0.39539999999999997</v>
+        <v>1.0643</v>
       </c>
       <c r="E23" s="7">
-        <v>5.79E-2</v>
+        <v>0.1172</v>
       </c>
       <c r="F23" s="7"/>
       <c r="G23" s="7"/>
       <c r="H23" s="15">
         <f t="shared" si="0"/>
-        <v>0.33749999999999997</v>
+        <v>0.94710000000000005</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -4229,23 +4244,23 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="19"/>
-      <c r="N10" s="19"/>
-      <c r="O10" s="19"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="22"/>
+      <c r="M10" s="22"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4257,7 +4272,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:R47"/>
+  <dimension ref="A1:T47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -4270,19 +4285,21 @@
     <col min="16" max="16" width="10" customWidth="1"/>
     <col min="17" max="17" width="11" customWidth="1"/>
     <col min="18" max="18" width="12" customWidth="1"/>
+    <col min="19" max="19" width="14" customWidth="1"/>
+    <col min="20" max="20" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>135</v>
       </c>
@@ -4290,7 +4307,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>34</v>
       </c>
@@ -4345,8 +4362,14 @@
       <c r="R5" s="5" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S5" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>45</v>
       </c>
@@ -4354,7 +4377,7 @@
         <v>46</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D6" s="7">
         <v>59996</v>
@@ -4398,14 +4421,22 @@
         <v>0</v>
       </c>
       <c r="Q6" s="7">
-        <v>0.67600000000000005</v>
+        <v>0.72799999999999998</v>
       </c>
       <c r="R6" s="15" t="str">
-        <f t="shared" ref="R6:R43" si="2">IFERROR(IF(M6&gt;$D$3,"Yes","No"),"")</f>
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+        <f t="shared" ref="R6:R43" si="2">IFERROR(IF(M6/S6&gt;$D$3,"Yes","No"),"")</f>
+        <v>No</v>
+      </c>
+      <c r="S6" s="15">
+        <f>Dataset!$J$2</f>
+        <v>421.23719999999997</v>
+      </c>
+      <c r="T6" s="18">
+        <f t="shared" ref="T6:T43" si="3">IFERROR(M6/S6*100,"")</f>
+        <v>0.45045570524160733</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>45</v>
       </c>
@@ -4413,7 +4444,7 @@
         <v>46</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D7" s="7">
         <v>59996</v>
@@ -4461,18 +4492,26 @@
       </c>
       <c r="R7" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+        <v>No</v>
+      </c>
+      <c r="S7" s="15">
+        <f>Dataset!$J$2</f>
+        <v>421.23719999999997</v>
+      </c>
+      <c r="T7" s="18">
+        <f t="shared" si="3"/>
+        <v>0.45045570524160733</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D8" s="7">
         <v>15000</v>
@@ -4516,22 +4555,30 @@
         <v>0</v>
       </c>
       <c r="Q8" s="7">
-        <v>0.127</v>
+        <v>0.14099999999999999</v>
       </c>
       <c r="R8" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+        <v>No</v>
+      </c>
+      <c r="S8" s="15">
+        <f>Dataset!$J$3</f>
+        <v>19.521100000000001</v>
+      </c>
+      <c r="T8" s="18">
+        <f t="shared" si="3"/>
+        <v>0.45465163336082492</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D9" s="7">
         <v>15000</v>
@@ -4579,10 +4626,18 @@
       </c>
       <c r="R9" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+        <v>No</v>
+      </c>
+      <c r="S9" s="15">
+        <f>Dataset!$J$3</f>
+        <v>19.521100000000001</v>
+      </c>
+      <c r="T9" s="18">
+        <f t="shared" si="3"/>
+        <v>0.45465163336082492</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>55</v>
       </c>
@@ -4590,7 +4645,7 @@
         <v>46</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D10" s="7">
         <v>130504</v>
@@ -4634,14 +4689,22 @@
         <v>0</v>
       </c>
       <c r="Q10" s="7">
-        <v>1.4039999999999999</v>
+        <v>1.4219999999999999</v>
       </c>
       <c r="R10" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+        <v>No</v>
+      </c>
+      <c r="S10" s="15">
+        <f>Dataset!$J$4</f>
+        <v>156.50190000000001</v>
+      </c>
+      <c r="T10" s="18">
+        <f t="shared" si="3"/>
+        <v>0.22999401285224014</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>55</v>
       </c>
@@ -4649,7 +4712,7 @@
         <v>46</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D11" s="7">
         <v>130504</v>
@@ -4693,14 +4756,22 @@
         <v>1</v>
       </c>
       <c r="Q11" s="7">
-        <v>0.33100000000000002</v>
+        <v>0.33200000000000002</v>
       </c>
       <c r="R11" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+        <v>No</v>
+      </c>
+      <c r="S11" s="15">
+        <f>Dataset!$J$4</f>
+        <v>156.50190000000001</v>
+      </c>
+      <c r="T11" s="18">
+        <f t="shared" si="3"/>
+        <v>0.22999401285224014</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>58</v>
       </c>
@@ -4708,7 +4779,7 @@
         <v>59</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D12" s="7">
         <v>1473</v>
@@ -4752,14 +4823,22 @@
         <v>0</v>
       </c>
       <c r="Q12" s="7">
-        <v>1.7000000000000001E-2</v>
+        <v>1.9E-2</v>
       </c>
       <c r="R12" s="15" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S12" s="15">
+        <f>Dataset!$J$5</f>
+        <v>1.2944</v>
+      </c>
+      <c r="T12" s="18">
+        <f t="shared" si="3"/>
+        <v>611.51529666254646</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>58</v>
       </c>
@@ -4767,7 +4846,7 @@
         <v>59</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D13" s="7">
         <v>1473</v>
@@ -4811,14 +4890,22 @@
         <v>3</v>
       </c>
       <c r="Q13" s="7">
-        <v>6.9000000000000006E-2</v>
+        <v>8.5999999999999993E-2</v>
       </c>
       <c r="R13" s="15" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S13" s="15">
+        <f>Dataset!$J$5</f>
+        <v>1.2944</v>
+      </c>
+      <c r="T13" s="18">
+        <f t="shared" si="3"/>
+        <v>11.388442521631644</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>62</v>
       </c>
@@ -4826,32 +4913,32 @@
         <v>59</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D14" s="7">
         <v>13790</v>
       </c>
       <c r="E14" s="7">
-        <v>1379</v>
+        <v>1376</v>
       </c>
       <c r="F14" s="14">
         <f t="shared" si="0"/>
-        <v>0.9</v>
+        <v>0.90021754894851336</v>
       </c>
       <c r="G14" s="7">
         <v>1.9303000000000001E-2</v>
       </c>
       <c r="H14" s="7">
-        <v>1.072E-3</v>
+        <v>1.0740000000000001E-3</v>
       </c>
       <c r="I14" s="7">
-        <v>4.1869999999999997E-3</v>
+        <v>4.1910000000000003E-3</v>
       </c>
       <c r="J14" s="7">
         <v>2.0695999999999999E-2</v>
       </c>
       <c r="K14" s="7">
-        <v>1.0579999999999999E-3</v>
+        <v>1.059E-3</v>
       </c>
       <c r="L14" s="7">
         <v>3.9490000000000003E-3</v>
@@ -4870,14 +4957,22 @@
         <v>0</v>
       </c>
       <c r="Q14" s="7">
-        <v>0.215</v>
+        <v>0.218</v>
       </c>
       <c r="R14" s="15" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S14" s="15">
+        <f>Dataset!$J$6</f>
+        <v>0.33339999999999997</v>
+      </c>
+      <c r="T14" s="18">
+        <f t="shared" si="3"/>
+        <v>6.2075584883023405</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>62</v>
       </c>
@@ -4885,58 +4980,66 @@
         <v>59</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D15" s="7">
         <v>13790</v>
       </c>
       <c r="E15" s="7">
-        <v>5093</v>
+        <v>5231</v>
       </c>
       <c r="F15" s="14">
         <f t="shared" si="0"/>
-        <v>0.63067440174039158</v>
+        <v>0.62066715010877449</v>
       </c>
       <c r="G15" s="7">
-        <v>6.9170000000000004E-3</v>
+        <v>7.9950000000000004E-3</v>
       </c>
       <c r="H15" s="7">
-        <v>3.5399999999999999E-4</v>
+        <v>4.0499999999999998E-4</v>
       </c>
       <c r="I15" s="7">
-        <v>1.508E-3</v>
+        <v>1.804E-3</v>
       </c>
       <c r="J15" s="7">
         <v>4.1469999999999996E-3</v>
       </c>
       <c r="K15" s="7">
-        <v>3.8699999999999997E-4</v>
+        <v>3.8999999999999999E-4</v>
       </c>
       <c r="L15" s="7">
-        <v>1.3320000000000001E-3</v>
+        <v>1.3600000000000001E-3</v>
       </c>
       <c r="M15" s="15">
         <f t="shared" si="1"/>
-        <v>6.9170000000000004E-3</v>
+        <v>7.9950000000000004E-3</v>
       </c>
       <c r="N15" s="7">
         <v>0</v>
       </c>
       <c r="O15" s="7">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="P15" s="7">
         <v>3</v>
       </c>
       <c r="Q15" s="7">
-        <v>0.78800000000000003</v>
+        <v>0.81</v>
       </c>
       <c r="R15" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>No</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+        <v>Yes</v>
+      </c>
+      <c r="S15" s="15">
+        <f>Dataset!$J$6</f>
+        <v>0.33339999999999997</v>
+      </c>
+      <c r="T15" s="18">
+        <f t="shared" si="3"/>
+        <v>2.3980203959208164</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>64</v>
       </c>
@@ -4944,32 +5047,32 @@
         <v>59</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D16" s="7">
         <v>2752</v>
       </c>
       <c r="E16" s="7">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F16" s="14">
         <f t="shared" si="0"/>
-        <v>0.90007267441860461</v>
+        <v>0.90079941860465118</v>
       </c>
       <c r="G16" s="7">
         <v>9.6729999999999993E-3</v>
       </c>
       <c r="H16" s="7">
-        <v>1.6570000000000001E-3</v>
+        <v>1.665E-3</v>
       </c>
       <c r="I16" s="7">
-        <v>4.8640000000000003E-3</v>
+        <v>4.8780000000000004E-3</v>
       </c>
       <c r="J16" s="7">
         <v>1.0291E-2</v>
       </c>
       <c r="K16" s="7">
-        <v>1.555E-3</v>
+        <v>1.557E-3</v>
       </c>
       <c r="L16" s="7">
         <v>4.725E-3</v>
@@ -4988,14 +5091,22 @@
         <v>0</v>
       </c>
       <c r="Q16" s="7">
-        <v>0.03</v>
+        <v>3.1E-2</v>
       </c>
       <c r="R16" s="15" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S16" s="15">
+        <f>Dataset!$J$7</f>
+        <v>0.1565</v>
+      </c>
+      <c r="T16" s="18">
+        <f t="shared" si="3"/>
+        <v>6.5757188498402552</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>64</v>
       </c>
@@ -5003,35 +5114,35 @@
         <v>59</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D17" s="7">
         <v>2752</v>
       </c>
       <c r="E17" s="7">
-        <v>2786</v>
+        <v>2790</v>
       </c>
       <c r="F17" s="14">
         <f t="shared" si="0"/>
-        <v>-1.2354651162790775E-2</v>
+        <v>-1.380813953488369E-2</v>
       </c>
       <c r="G17" s="7">
         <v>1.918E-3</v>
       </c>
       <c r="H17" s="7">
-        <v>2.1999999999999999E-5</v>
+        <v>2.0999999999999999E-5</v>
       </c>
       <c r="I17" s="7">
-        <v>1.2E-4</v>
+        <v>1.0399999999999999E-4</v>
       </c>
       <c r="J17" s="7">
         <v>1.024E-3</v>
       </c>
       <c r="K17" s="7">
-        <v>1.1E-5</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="L17" s="7">
-        <v>3.6999999999999998E-5</v>
+        <v>3.4999999999999997E-5</v>
       </c>
       <c r="M17" s="15">
         <f t="shared" si="1"/>
@@ -5041,20 +5152,28 @@
         <v>0</v>
       </c>
       <c r="O17" s="7">
-        <v>989</v>
+        <v>993</v>
       </c>
       <c r="P17" s="7">
         <v>3</v>
       </c>
       <c r="Q17" s="7">
-        <v>0.1</v>
+        <v>0.112</v>
       </c>
       <c r="R17" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>No</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+        <v>Yes</v>
+      </c>
+      <c r="S17" s="15">
+        <f>Dataset!$J$7</f>
+        <v>0.1565</v>
+      </c>
+      <c r="T17" s="18">
+        <f t="shared" si="3"/>
+        <v>1.22555910543131</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>66</v>
       </c>
@@ -5062,7 +5181,7 @@
         <v>67</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D18" s="7">
         <v>3410</v>
@@ -5106,14 +5225,22 @@
         <v>0</v>
       </c>
       <c r="Q18" s="7">
-        <v>3.6999999999999998E-2</v>
+        <v>0.04</v>
       </c>
       <c r="R18" s="15" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S18" s="15">
+        <f>Dataset!$J$8</f>
+        <v>0.8175</v>
+      </c>
+      <c r="T18" s="18">
+        <f t="shared" si="3"/>
+        <v>14.789847094801223</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>66</v>
       </c>
@@ -5121,26 +5248,26 @@
         <v>67</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D19" s="7">
         <v>3410</v>
       </c>
       <c r="E19" s="7">
-        <v>1068</v>
+        <v>1066</v>
       </c>
       <c r="F19" s="14">
         <f t="shared" si="0"/>
-        <v>0.68680351906158355</v>
+        <v>0.68739002932551319</v>
       </c>
       <c r="G19" s="7">
         <v>6.2509999999999996E-3</v>
       </c>
       <c r="H19" s="7">
-        <v>6.29E-4</v>
+        <v>6.3000000000000003E-4</v>
       </c>
       <c r="I19" s="7">
-        <v>2.7190000000000001E-3</v>
+        <v>2.7200000000000002E-3</v>
       </c>
       <c r="J19" s="7">
         <v>6.8649999999999996E-3</v>
@@ -5171,8 +5298,16 @@
         <f t="shared" si="2"/>
         <v>No</v>
       </c>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S19" s="15">
+        <f>Dataset!$J$8</f>
+        <v>0.8175</v>
+      </c>
+      <c r="T19" s="18">
+        <f t="shared" si="3"/>
+        <v>0.83975535168195714</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>69</v>
       </c>
@@ -5180,7 +5315,7 @@
         <v>67</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D20" s="7">
         <v>2926</v>
@@ -5224,14 +5359,22 @@
         <v>0</v>
       </c>
       <c r="Q20" s="7">
-        <v>3.9E-2</v>
+        <v>3.6999999999999998E-2</v>
       </c>
       <c r="R20" s="15" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S20" s="15">
+        <f>Dataset!$J$9</f>
+        <v>0.26540000000000002</v>
+      </c>
+      <c r="T20" s="18">
+        <f t="shared" si="3"/>
+        <v>17.108892238131123</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>69</v>
       </c>
@@ -5239,26 +5382,26 @@
         <v>67</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D21" s="7">
         <v>2926</v>
       </c>
       <c r="E21" s="7">
-        <v>2729</v>
+        <v>2730</v>
       </c>
       <c r="F21" s="14">
         <f t="shared" si="0"/>
-        <v>6.7327409432672569E-2</v>
+        <v>6.6985645933014371E-2</v>
       </c>
       <c r="G21" s="7">
         <v>1.3249E-2</v>
       </c>
       <c r="H21" s="7">
-        <v>3.3799999999999998E-4</v>
+        <v>3.3399999999999999E-4</v>
       </c>
       <c r="I21" s="7">
-        <v>1.928E-3</v>
+        <v>1.8649999999999999E-3</v>
       </c>
       <c r="J21" s="7">
         <v>3.009E-3</v>
@@ -5283,14 +5426,22 @@
         <v>3</v>
       </c>
       <c r="Q21" s="7">
-        <v>0.11600000000000001</v>
+        <v>0.129</v>
       </c>
       <c r="R21" s="15" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S21" s="15">
+        <f>Dataset!$J$9</f>
+        <v>0.26540000000000002</v>
+      </c>
+      <c r="T21" s="18">
+        <f t="shared" si="3"/>
+        <v>4.992087415222306</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>71</v>
       </c>
@@ -5298,35 +5449,35 @@
         <v>72</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D22" s="7">
         <v>211874</v>
       </c>
       <c r="E22" s="7">
-        <v>21187</v>
+        <v>21172</v>
       </c>
       <c r="F22" s="14">
         <f t="shared" si="0"/>
-        <v>0.90000188791451519</v>
+        <v>0.90007268470883639</v>
       </c>
       <c r="G22" s="7">
         <v>4.7434999999999998E-2</v>
       </c>
       <c r="H22" s="7">
-        <v>5.5199999999999997E-4</v>
+        <v>5.4799999999999998E-4</v>
       </c>
       <c r="I22" s="7">
-        <v>2.3280000000000002E-3</v>
+        <v>2.3040000000000001E-3</v>
       </c>
       <c r="J22" s="7">
         <v>5.0117000000000002E-2</v>
       </c>
       <c r="K22" s="7">
-        <v>3.4740000000000001E-3</v>
+        <v>3.483E-3</v>
       </c>
       <c r="L22" s="7">
-        <v>1.7767999999999999E-2</v>
+        <v>1.7822999999999999E-2</v>
       </c>
       <c r="M22" s="15">
         <f t="shared" si="1"/>
@@ -5342,14 +5493,22 @@
         <v>0</v>
       </c>
       <c r="Q22" s="7">
-        <v>2.609</v>
+        <v>2.7069999999999999</v>
       </c>
       <c r="R22" s="15" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S22" s="15">
+        <f>Dataset!$J$10</f>
+        <v>2.2942</v>
+      </c>
+      <c r="T22" s="18">
+        <f t="shared" si="3"/>
+        <v>2.184508761223956</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>71</v>
       </c>
@@ -5357,58 +5516,66 @@
         <v>72</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D23" s="7">
         <v>211874</v>
       </c>
       <c r="E23" s="7">
-        <v>44530</v>
+        <v>42555</v>
       </c>
       <c r="F23" s="14">
         <f t="shared" si="0"/>
-        <v>0.78982791659193674</v>
+        <v>0.79914949451088857</v>
       </c>
       <c r="G23" s="7">
-        <v>5.8889999999999998E-2</v>
+        <v>5.5662999999999997E-2</v>
       </c>
       <c r="H23" s="7">
-        <v>7.4899999999999999E-4</v>
+        <v>7.6000000000000004E-4</v>
       </c>
       <c r="I23" s="7">
-        <v>3.6779999999999998E-3</v>
+        <v>3.7959999999999999E-3</v>
       </c>
       <c r="J23" s="7">
         <v>2.1922000000000001E-2</v>
       </c>
       <c r="K23" s="7">
-        <v>1.4009999999999999E-3</v>
+        <v>1.407E-3</v>
       </c>
       <c r="L23" s="7">
-        <v>5.8230000000000001E-3</v>
+        <v>5.9709999999999997E-3</v>
       </c>
       <c r="M23" s="15">
         <f t="shared" si="1"/>
-        <v>5.8889999999999998E-2</v>
+        <v>5.5662999999999997E-2</v>
       </c>
       <c r="N23" s="7">
         <v>0</v>
       </c>
       <c r="O23" s="7">
-        <v>4422</v>
+        <v>4149</v>
       </c>
       <c r="P23" s="7">
         <v>3</v>
       </c>
       <c r="Q23" s="7">
-        <v>9.5950000000000006</v>
+        <v>9.923</v>
       </c>
       <c r="R23" s="15" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S23" s="15">
+        <f>Dataset!$J$10</f>
+        <v>2.2942</v>
+      </c>
+      <c r="T23" s="18">
+        <f t="shared" si="3"/>
+        <v>2.4262488013250807</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>75</v>
       </c>
@@ -5416,35 +5583,35 @@
         <v>72</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D24" s="7">
         <v>446670</v>
       </c>
       <c r="E24" s="7">
-        <v>44667</v>
+        <v>44633</v>
       </c>
       <c r="F24" s="14">
         <f t="shared" si="0"/>
-        <v>0.9</v>
+        <v>0.9000761188349341</v>
       </c>
       <c r="G24" s="7">
         <v>2.4506E-2</v>
       </c>
       <c r="H24" s="7">
-        <v>3.7599999999999998E-4</v>
+        <v>3.7500000000000001E-4</v>
       </c>
       <c r="I24" s="7">
-        <v>1.4400000000000001E-3</v>
+        <v>1.4350000000000001E-3</v>
       </c>
       <c r="J24" s="7">
         <v>3.6756999999999998E-2</v>
       </c>
       <c r="K24" s="7">
-        <v>1.137E-3</v>
+        <v>1.1379999999999999E-3</v>
       </c>
       <c r="L24" s="7">
-        <v>4.7869999999999996E-3</v>
+        <v>4.7889999999999999E-3</v>
       </c>
       <c r="M24" s="15">
         <f t="shared" si="1"/>
@@ -5460,14 +5627,22 @@
         <v>0</v>
       </c>
       <c r="Q24" s="7">
-        <v>5.7130000000000001</v>
+        <v>5.7249999999999996</v>
       </c>
       <c r="R24" s="15" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S24" s="15">
+        <f>Dataset!$J$11</f>
+        <v>1.8779999999999999</v>
+      </c>
+      <c r="T24" s="18">
+        <f t="shared" si="3"/>
+        <v>1.9572417465388712</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>75</v>
       </c>
@@ -5475,58 +5650,66 @@
         <v>72</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D25" s="7">
         <v>446670</v>
       </c>
       <c r="E25" s="7">
-        <v>85018</v>
+        <v>150195</v>
       </c>
       <c r="F25" s="14">
         <f t="shared" si="0"/>
-        <v>0.80966261445810106</v>
+        <v>0.66374504667875611</v>
       </c>
       <c r="G25" s="7">
-        <v>4.6064000000000001E-2</v>
+        <v>0.221384</v>
       </c>
       <c r="H25" s="7">
-        <v>8.6300000000000005E-4</v>
+        <v>1.9595999999999999E-2</v>
       </c>
       <c r="I25" s="7">
-        <v>4.0369999999999998E-3</v>
+        <v>0.15328600000000001</v>
       </c>
       <c r="J25" s="7">
-        <v>1.7166000000000001E-2</v>
+        <v>1.8332000000000001E-2</v>
       </c>
       <c r="K25" s="7">
-        <v>8.3500000000000002E-4</v>
+        <v>6.9999999999999999E-4</v>
       </c>
       <c r="L25" s="7">
-        <v>3.6020000000000002E-3</v>
+        <v>3.1199999999999999E-3</v>
       </c>
       <c r="M25" s="15">
         <f t="shared" si="1"/>
-        <v>4.6064000000000001E-2</v>
+        <v>0.221384</v>
       </c>
       <c r="N25" s="7">
         <v>0</v>
       </c>
       <c r="O25" s="7">
-        <v>3987</v>
+        <v>15225</v>
       </c>
       <c r="P25" s="7">
         <v>3</v>
       </c>
       <c r="Q25" s="7">
-        <v>27.832000000000001</v>
+        <v>140.315</v>
       </c>
       <c r="R25" s="15" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S25" s="15">
+        <f>Dataset!$J$11</f>
+        <v>1.8779999999999999</v>
+      </c>
+      <c r="T25" s="18">
+        <f t="shared" si="3"/>
+        <v>11.78828541001065</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>78</v>
       </c>
@@ -5534,17 +5717,17 @@
         <v>72</v>
       </c>
       <c r="C26" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D26">
         <v>108958</v>
       </c>
       <c r="E26">
-        <v>10894</v>
+        <v>10890</v>
       </c>
       <c r="F26">
         <f t="shared" si="0"/>
-        <v>0.90001652012702138</v>
+        <v>0.9000532315204024</v>
       </c>
       <c r="G26">
         <v>2.859E-3</v>
@@ -5578,14 +5761,22 @@
         <v>0</v>
       </c>
       <c r="Q26">
-        <v>1.2649999999999999</v>
+        <v>1.2390000000000001</v>
       </c>
       <c r="R26" t="str">
         <f t="shared" si="2"/>
         <v>No</v>
       </c>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S26" s="19">
+        <f>Dataset!$J$12</f>
+        <v>1.6142000000000001</v>
+      </c>
+      <c r="T26" s="20">
+        <f t="shared" si="3"/>
+        <v>0.23423367612439597</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
         <v>78</v>
       </c>
@@ -5593,17 +5784,17 @@
         <v>72</v>
       </c>
       <c r="C27" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D27">
         <v>108958</v>
       </c>
       <c r="E27">
-        <v>10894</v>
+        <v>10890</v>
       </c>
       <c r="F27">
         <f t="shared" si="0"/>
-        <v>0.90001652012702138</v>
+        <v>0.9000532315204024</v>
       </c>
       <c r="G27">
         <v>2.859E-3</v>
@@ -5637,14 +5828,22 @@
         <v>1</v>
       </c>
       <c r="Q27">
-        <v>0.34799999999999998</v>
+        <v>0.34499999999999997</v>
       </c>
       <c r="R27" t="str">
         <f t="shared" si="2"/>
         <v>No</v>
       </c>
-    </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S27" s="19">
+        <f>Dataset!$J$12</f>
+        <v>1.6142000000000001</v>
+      </c>
+      <c r="T27" s="20">
+        <f t="shared" si="3"/>
+        <v>0.23423367612439597</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
         <v>80</v>
       </c>
@@ -5652,17 +5851,17 @@
         <v>72</v>
       </c>
       <c r="C28" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D28">
         <v>405680</v>
       </c>
       <c r="E28">
-        <v>40568</v>
+        <v>40563</v>
       </c>
       <c r="F28">
         <f t="shared" si="0"/>
-        <v>0.9</v>
+        <v>0.90001232498521</v>
       </c>
       <c r="G28">
         <v>2.0625000000000001E-2</v>
@@ -5671,7 +5870,7 @@
         <v>9.8999999999999999E-4</v>
       </c>
       <c r="I28">
-        <v>3.8479999999999999E-3</v>
+        <v>3.8470000000000002E-3</v>
       </c>
       <c r="J28">
         <v>5.0375999999999997E-2</v>
@@ -5680,7 +5879,7 @@
         <v>1.4059999999999999E-3</v>
       </c>
       <c r="L28">
-        <v>4.9979999999999998E-3</v>
+        <v>4.999E-3</v>
       </c>
       <c r="M28">
         <f t="shared" si="1"/>
@@ -5696,14 +5895,22 @@
         <v>0</v>
       </c>
       <c r="Q28">
-        <v>8.15</v>
+        <v>8.0739999999999998</v>
       </c>
       <c r="R28" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S28" s="19">
+        <f>Dataset!$J$13</f>
+        <v>4.8654000000000002</v>
+      </c>
+      <c r="T28" s="20">
+        <f t="shared" si="3"/>
+        <v>1.0353927734615858</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
         <v>80</v>
       </c>
@@ -5711,58 +5918,66 @@
         <v>72</v>
       </c>
       <c r="C29" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D29">
         <v>405680</v>
       </c>
       <c r="E29">
-        <v>90425</v>
+        <v>98032</v>
       </c>
       <c r="F29">
         <f t="shared" si="0"/>
-        <v>0.77710264247682903</v>
+        <v>0.75835140997830797</v>
       </c>
       <c r="G29">
-        <v>0.38563599999999998</v>
+        <v>0.36501400000000001</v>
       </c>
       <c r="H29">
-        <v>7.4250000000000002E-3</v>
+        <v>1.3302E-2</v>
       </c>
       <c r="I29">
-        <v>2.6195E-2</v>
+        <v>0.108886</v>
       </c>
       <c r="J29">
-        <v>3.5486999999999998E-2</v>
+        <v>3.5890999999999999E-2</v>
       </c>
       <c r="K29">
-        <v>1.0640000000000001E-3</v>
+        <v>1.0380000000000001E-3</v>
       </c>
       <c r="L29">
-        <v>3.9360000000000003E-3</v>
+        <v>3.859E-3</v>
       </c>
       <c r="M29">
         <f t="shared" si="1"/>
-        <v>0.38563599999999998</v>
+        <v>0.36501400000000001</v>
       </c>
       <c r="N29">
         <v>0</v>
       </c>
       <c r="O29">
-        <v>2808</v>
+        <v>4044</v>
       </c>
       <c r="P29">
         <v>3</v>
       </c>
       <c r="Q29">
-        <v>54.451999999999998</v>
+        <v>80.122</v>
       </c>
       <c r="R29" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S29" s="19">
+        <f>Dataset!$J$13</f>
+        <v>4.8654000000000002</v>
+      </c>
+      <c r="T29" s="20">
+        <f t="shared" si="3"/>
+        <v>7.5022403091215519</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>83</v>
       </c>
@@ -5770,7 +5985,7 @@
         <v>84</v>
       </c>
       <c r="C30" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D30">
         <v>5912</v>
@@ -5814,14 +6029,22 @@
         <v>0</v>
       </c>
       <c r="Q30">
-        <v>5.6000000000000001E-2</v>
+        <v>6.0999999999999999E-2</v>
       </c>
       <c r="R30" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S30" s="19">
+        <f>Dataset!$J$14</f>
+        <v>0.23269999999999999</v>
+      </c>
+      <c r="T30" s="20">
+        <f t="shared" si="3"/>
+        <v>8.7847013321873657</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>83</v>
       </c>
@@ -5829,26 +6052,26 @@
         <v>84</v>
       </c>
       <c r="C31" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D31">
         <v>5912</v>
       </c>
       <c r="E31">
-        <v>5230</v>
+        <v>5129</v>
       </c>
       <c r="F31">
         <f t="shared" si="0"/>
-        <v>0.11535859269282811</v>
+        <v>0.13244248985115026</v>
       </c>
       <c r="G31">
-        <v>7.9150000000000002E-3</v>
+        <v>8.3280000000000003E-3</v>
       </c>
       <c r="H31">
-        <v>3.0400000000000002E-4</v>
+        <v>2.72E-4</v>
       </c>
       <c r="I31">
-        <v>2.1940000000000002E-3</v>
+        <v>1.6739999999999999E-3</v>
       </c>
       <c r="J31">
         <v>2.3149999999999998E-3</v>
@@ -5857,30 +6080,38 @@
         <v>2.6400000000000002E-4</v>
       </c>
       <c r="L31">
-        <v>1.333E-3</v>
+        <v>1.3339999999999999E-3</v>
       </c>
       <c r="M31">
         <f t="shared" si="1"/>
-        <v>7.9150000000000002E-3</v>
+        <v>8.3280000000000003E-3</v>
       </c>
       <c r="N31">
         <v>0</v>
       </c>
       <c r="O31">
-        <v>10389</v>
+        <v>10386</v>
       </c>
       <c r="P31">
         <v>3</v>
       </c>
       <c r="Q31">
-        <v>0.245</v>
+        <v>0.26700000000000002</v>
       </c>
       <c r="R31" t="str">
         <f t="shared" si="2"/>
-        <v>No</v>
-      </c>
-    </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+        <v>Yes</v>
+      </c>
+      <c r="S31" s="19">
+        <f>Dataset!$J$14</f>
+        <v>0.23269999999999999</v>
+      </c>
+      <c r="T31" s="20">
+        <f t="shared" si="3"/>
+        <v>3.5788568972926518</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>88</v>
       </c>
@@ -5888,7 +6119,7 @@
         <v>84</v>
       </c>
       <c r="C32" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D32">
         <v>16694</v>
@@ -5932,14 +6163,22 @@
         <v>0</v>
       </c>
       <c r="Q32">
-        <v>0.19</v>
+        <v>0.18099999999999999</v>
       </c>
       <c r="R32" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S32" s="19">
+        <f>Dataset!$J$15</f>
+        <v>0.3029</v>
+      </c>
+      <c r="T32" s="20">
+        <f t="shared" si="3"/>
+        <v>7.1591284252228453</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>88</v>
       </c>
@@ -5947,26 +6186,26 @@
         <v>84</v>
       </c>
       <c r="C33" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D33">
         <v>16694</v>
       </c>
       <c r="E33">
-        <v>11981</v>
+        <v>11921</v>
       </c>
       <c r="F33">
         <f t="shared" si="0"/>
-        <v>0.28231700011980354</v>
+        <v>0.28591110578651013</v>
       </c>
       <c r="G33">
         <v>6.045E-3</v>
       </c>
       <c r="H33">
-        <v>1.12E-4</v>
+        <v>1.11E-4</v>
       </c>
       <c r="I33">
-        <v>6.11E-4</v>
+        <v>5.9199999999999997E-4</v>
       </c>
       <c r="J33">
         <v>3.0230000000000001E-3</v>
@@ -5991,14 +6230,22 @@
         <v>3</v>
       </c>
       <c r="Q33">
-        <v>0.66200000000000003</v>
+        <v>0.70399999999999996</v>
       </c>
       <c r="R33" t="str">
         <f t="shared" si="2"/>
-        <v>No</v>
-      </c>
-    </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+        <v>Yes</v>
+      </c>
+      <c r="S33" s="19">
+        <f>Dataset!$J$15</f>
+        <v>0.3029</v>
+      </c>
+      <c r="T33" s="20">
+        <f t="shared" si="3"/>
+        <v>1.9957081545064377</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>90</v>
       </c>
@@ -6006,26 +6253,26 @@
         <v>84</v>
       </c>
       <c r="C34" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D34">
         <v>63998</v>
       </c>
       <c r="E34">
-        <v>6398</v>
+        <v>6378</v>
       </c>
       <c r="F34">
         <f t="shared" si="0"/>
-        <v>0.90002812587893377</v>
+        <v>0.90034063564486388</v>
       </c>
       <c r="G34">
         <v>4.0090000000000004E-3</v>
       </c>
       <c r="H34">
-        <v>3.6400000000000001E-4</v>
+        <v>3.6299999999999999E-4</v>
       </c>
       <c r="I34">
-        <v>1.333E-3</v>
+        <v>1.3309999999999999E-3</v>
       </c>
       <c r="J34">
         <v>5.1440000000000001E-3</v>
@@ -6050,14 +6297,22 @@
         <v>0</v>
       </c>
       <c r="Q34">
-        <v>0.66</v>
+        <v>0.64600000000000002</v>
       </c>
       <c r="R34" t="str">
         <f t="shared" si="2"/>
-        <v>No</v>
-      </c>
-    </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+        <v>Yes</v>
+      </c>
+      <c r="S34" s="19">
+        <f>Dataset!$J$16</f>
+        <v>0.45639999999999997</v>
+      </c>
+      <c r="T34" s="20">
+        <f t="shared" si="3"/>
+        <v>1.1270815074496057</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>90</v>
       </c>
@@ -6065,17 +6320,17 @@
         <v>84</v>
       </c>
       <c r="C35" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D35">
         <v>63998</v>
       </c>
       <c r="E35">
-        <v>6536</v>
+        <v>6530</v>
       </c>
       <c r="F35">
         <f t="shared" si="0"/>
-        <v>0.89787180849401538</v>
+        <v>0.89796556142379447</v>
       </c>
       <c r="G35">
         <v>4.0090000000000004E-3</v>
@@ -6109,14 +6364,22 @@
         <v>2</v>
       </c>
       <c r="Q35">
-        <v>0.82</v>
+        <v>0.81</v>
       </c>
       <c r="R35" t="str">
         <f t="shared" si="2"/>
         <v>No</v>
       </c>
-    </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S35" s="19">
+        <f>Dataset!$J$16</f>
+        <v>0.45639999999999997</v>
+      </c>
+      <c r="T35" s="20">
+        <f t="shared" si="3"/>
+        <v>0.92703768624014038</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>93</v>
       </c>
@@ -6124,7 +6387,7 @@
         <v>84</v>
       </c>
       <c r="C36" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D36">
         <v>69451</v>
@@ -6168,14 +6431,22 @@
         <v>0</v>
       </c>
       <c r="Q36">
-        <v>0.502</v>
+        <v>0.48299999999999998</v>
       </c>
       <c r="R36" t="str">
         <f t="shared" si="2"/>
         <v>No</v>
       </c>
-    </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S36" s="19">
+        <f>Dataset!$J$17</f>
+        <v>0.25019999999999998</v>
+      </c>
+      <c r="T36" s="20">
+        <f t="shared" si="3"/>
+        <v>0.16706634692246206</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>93</v>
       </c>
@@ -6183,7 +6454,7 @@
         <v>84</v>
       </c>
       <c r="C37" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D37">
         <v>69451</v>
@@ -6227,14 +6498,22 @@
         <v>1</v>
       </c>
       <c r="Q37">
-        <v>0.17</v>
+        <v>0.159</v>
       </c>
       <c r="R37" t="str">
         <f t="shared" si="2"/>
         <v>No</v>
       </c>
-    </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S37" s="19">
+        <f>Dataset!$J$17</f>
+        <v>0.25019999999999998</v>
+      </c>
+      <c r="T37" s="20">
+        <f t="shared" si="3"/>
+        <v>0.16706634692246206</v>
+      </c>
+    </row>
+    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>97</v>
       </c>
@@ -6242,7 +6521,7 @@
         <v>84</v>
       </c>
       <c r="C38" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D38">
         <v>345944</v>
@@ -6286,14 +6565,22 @@
         <v>0</v>
       </c>
       <c r="Q38">
-        <v>3.9089999999999998</v>
+        <v>3.863</v>
       </c>
       <c r="R38" t="str">
         <f t="shared" si="2"/>
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+        <v>No</v>
+      </c>
+      <c r="S38" s="19">
+        <f>Dataset!$J$18</f>
+        <v>228.80369999999999</v>
+      </c>
+      <c r="T38" s="20">
+        <f t="shared" si="3"/>
+        <v>7.6476910119897545E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>97</v>
       </c>
@@ -6301,7 +6588,7 @@
         <v>84</v>
       </c>
       <c r="C39" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D39">
         <v>345944</v>
@@ -6345,14 +6632,22 @@
         <v>1</v>
       </c>
       <c r="Q39">
-        <v>1.514</v>
+        <v>1.4970000000000001</v>
       </c>
       <c r="R39" t="str">
         <f t="shared" si="2"/>
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+        <v>No</v>
+      </c>
+      <c r="S39" s="19">
+        <f>Dataset!$J$18</f>
+        <v>228.80369999999999</v>
+      </c>
+      <c r="T39" s="20">
+        <f t="shared" si="3"/>
+        <v>7.6476910119897545E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>99</v>
       </c>
@@ -6360,7 +6655,7 @@
         <v>100</v>
       </c>
       <c r="C40" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D40">
         <v>1869988</v>
@@ -6404,14 +6699,22 @@
         <v>0</v>
       </c>
       <c r="Q40">
-        <v>25.905999999999999</v>
+        <v>25.439</v>
       </c>
       <c r="R40" t="str">
         <f t="shared" si="2"/>
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+        <v>No</v>
+      </c>
+      <c r="S40" s="19">
+        <f>Dataset!$J$19</f>
+        <v>2.3605999999999998</v>
+      </c>
+      <c r="T40" s="20">
+        <f t="shared" si="3"/>
+        <v>0.79640769295941716</v>
+      </c>
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>99</v>
       </c>
@@ -6419,7 +6722,7 @@
         <v>100</v>
       </c>
       <c r="C41" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D41">
         <v>1869988</v>
@@ -6463,14 +6766,22 @@
         <v>1</v>
       </c>
       <c r="Q41">
-        <v>12.752000000000001</v>
+        <v>12.962</v>
       </c>
       <c r="R41" t="str">
         <f t="shared" si="2"/>
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+        <v>No</v>
+      </c>
+      <c r="S41" s="19">
+        <f>Dataset!$J$19</f>
+        <v>2.3605999999999998</v>
+      </c>
+      <c r="T41" s="20">
+        <f t="shared" si="3"/>
+        <v>0.79640769295941716</v>
+      </c>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>104</v>
       </c>
@@ -6478,7 +6789,7 @@
         <v>100</v>
       </c>
       <c r="C42" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D42">
         <v>31400</v>
@@ -6522,14 +6833,22 @@
         <v>0</v>
       </c>
       <c r="Q42">
-        <v>0.35899999999999999</v>
+        <v>0.35799999999999998</v>
       </c>
       <c r="R42" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S42" s="19">
+        <f>Dataset!$J$20</f>
+        <v>2.4527999999999999</v>
+      </c>
+      <c r="T42" s="20">
+        <f t="shared" si="3"/>
+        <v>5.2516715590345733</v>
+      </c>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>104</v>
       </c>
@@ -6537,78 +6856,86 @@
         <v>100</v>
       </c>
       <c r="C43" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D43">
         <v>31400</v>
       </c>
       <c r="E43">
-        <v>25128</v>
+        <v>24908</v>
       </c>
       <c r="F43">
         <f t="shared" si="0"/>
-        <v>0.19974522292993635</v>
+        <v>0.20675159235668794</v>
       </c>
       <c r="G43">
-        <v>0.15196999999999999</v>
+        <v>0.151949</v>
       </c>
       <c r="H43">
-        <v>2.529E-3</v>
+        <v>2.496E-3</v>
       </c>
       <c r="I43">
-        <v>1.4290000000000001E-2</v>
+        <v>1.4452E-2</v>
       </c>
       <c r="J43">
         <v>2.7682999999999999E-2</v>
       </c>
       <c r="K43">
-        <v>3.0049999999999999E-3</v>
+        <v>2.9610000000000001E-3</v>
       </c>
       <c r="L43">
-        <v>1.3150999999999999E-2</v>
+        <v>1.3044999999999999E-2</v>
       </c>
       <c r="M43">
         <f t="shared" si="1"/>
-        <v>0.15196999999999999</v>
+        <v>0.151949</v>
       </c>
       <c r="N43">
         <v>0</v>
       </c>
       <c r="O43">
-        <v>46108</v>
+        <v>46048</v>
       </c>
       <c r="P43">
         <v>3</v>
       </c>
       <c r="Q43">
-        <v>2.472</v>
+        <v>2.556</v>
       </c>
       <c r="R43" t="str">
         <f t="shared" si="2"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S43" s="19">
+        <f>Dataset!$J$20</f>
+        <v>2.4527999999999999</v>
+      </c>
+      <c r="T43" s="20">
+        <f t="shared" si="3"/>
+        <v>6.1949200913242013</v>
+      </c>
+    </row>
+    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B46" t="str">
         <f>COUNTIFS(C6:C43,"No refinement",R6:R43,"Yes")&amp;"/"&amp;COUNTIF(C6:C43,"No refinement")</f>
-        <v>16/19</v>
-      </c>
-    </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+        <v>12/19</v>
+      </c>
+    </row>
+    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B47" t="str">
         <f>COUNTIFS(C6:C43,"Bidirectional refinement",R6:R43,"Yes")&amp;"/"&amp;COUNTIF(C6:C43,"Bidirectional refinement")</f>
-        <v>11/19</v>
+        <v>10/19</v>
       </c>
     </row>
   </sheetData>
@@ -6628,12 +6955,12 @@
   <sheetData>
     <row r="1" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -6647,67 +6974,67 @@
         <v>110</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="V4" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="X4" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
@@ -7041,12 +7368,12 @@
   <sheetData>
     <row r="1" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7054,7 +7381,7 @@
         <v>34</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>110</v>
@@ -7069,16 +7396,16 @@
         <v>143</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -7092,26 +7419,26 @@
         <v>13790</v>
       </c>
       <c r="D5" s="7">
-        <v>13446</v>
+        <v>13346</v>
       </c>
       <c r="E5" s="14">
         <f t="shared" ref="E5:E29" si="0">IFERROR(1-D5/C5,"")</f>
-        <v>2.4945612762871661E-2</v>
+        <v>3.2197244379985501E-2</v>
       </c>
       <c r="F5" s="7">
         <v>3</v>
       </c>
       <c r="G5" s="7">
-        <v>4761</v>
+        <v>4757</v>
       </c>
       <c r="H5" s="7">
-        <v>4.1000000000000003E-3</v>
+        <v>4.065E-3</v>
       </c>
       <c r="I5" s="7">
-        <v>4.3999999999999999E-5</v>
+        <v>4.5000000000000003E-5</v>
       </c>
       <c r="J5" s="7">
-        <v>2.9E-4</v>
+        <v>2.9399999999999999E-4</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -7125,11 +7452,11 @@
         <v>13790</v>
       </c>
       <c r="D6" s="7">
-        <v>8238</v>
+        <v>9089</v>
       </c>
       <c r="E6" s="14">
         <f t="shared" si="0"/>
-        <v>0.40261058738216093</v>
+        <v>0.34089920232052207</v>
       </c>
       <c r="F6" s="7">
         <v>3</v>
@@ -7138,13 +7465,13 @@
         <v>2301</v>
       </c>
       <c r="H6" s="7">
-        <v>4.7590000000000002E-3</v>
+        <v>1.7493000000000002E-2</v>
       </c>
       <c r="I6" s="7">
-        <v>1.64E-4</v>
+        <v>2.3900000000000001E-4</v>
       </c>
       <c r="J6" s="7">
-        <v>7.9299999999999998E-4</v>
+        <v>9.3199999999999999E-4</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -7158,26 +7485,26 @@
         <v>13790</v>
       </c>
       <c r="D7" s="7">
-        <v>5093</v>
+        <v>5231</v>
       </c>
       <c r="E7" s="14">
         <f t="shared" si="0"/>
-        <v>0.63067440174039158</v>
+        <v>0.62066715010877449</v>
       </c>
       <c r="F7" s="7">
         <v>3</v>
       </c>
       <c r="G7" s="7">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="H7" s="7">
-        <v>6.9170000000000004E-3</v>
+        <v>7.9950000000000004E-3</v>
       </c>
       <c r="I7" s="7">
-        <v>3.7800000000000003E-4</v>
+        <v>3.9399999999999998E-4</v>
       </c>
       <c r="J7" s="7">
-        <v>1.377E-3</v>
+        <v>1.4450000000000001E-3</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -7191,26 +7518,26 @@
         <v>13790</v>
       </c>
       <c r="D8" s="7">
-        <v>3799</v>
+        <v>3672</v>
       </c>
       <c r="E8" s="14">
         <f t="shared" si="0"/>
-        <v>0.72451051486584483</v>
+        <v>0.73372008701957947</v>
       </c>
       <c r="F8" s="7">
         <v>3</v>
       </c>
       <c r="G8" s="7">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="H8" s="7">
-        <v>1.4095999999999999E-2</v>
+        <v>1.0472E-2</v>
       </c>
       <c r="I8" s="7">
-        <v>5.8600000000000004E-4</v>
+        <v>5.6899999999999995E-4</v>
       </c>
       <c r="J8" s="7">
-        <v>2.0279999999999999E-3</v>
+        <v>2.0209999999999998E-3</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -7224,26 +7551,26 @@
         <v>13790</v>
       </c>
       <c r="D9" s="7">
-        <v>2949</v>
+        <v>2874</v>
       </c>
       <c r="E9" s="14">
         <f t="shared" si="0"/>
-        <v>0.78614938361131248</v>
+        <v>0.79158810732414797</v>
       </c>
       <c r="F9" s="7">
         <v>3</v>
       </c>
       <c r="G9" s="7">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H9" s="7">
-        <v>1.5252E-2</v>
+        <v>1.9372E-2</v>
       </c>
       <c r="I9" s="7">
-        <v>8.9400000000000005E-4</v>
+        <v>9.2000000000000003E-4</v>
       </c>
       <c r="J9" s="7">
-        <v>3.339E-3</v>
+        <v>3.5620000000000001E-3</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -7257,26 +7584,26 @@
         <v>211874</v>
       </c>
       <c r="D10" s="7">
-        <v>85349</v>
+        <v>96954</v>
       </c>
       <c r="E10" s="14">
         <f t="shared" si="0"/>
-        <v>0.59717096009892678</v>
+        <v>0.54239784022579451</v>
       </c>
       <c r="F10" s="7">
         <v>3</v>
       </c>
       <c r="G10" s="7">
-        <v>22684</v>
+        <v>24710</v>
       </c>
       <c r="H10" s="7">
-        <v>8.5232000000000002E-2</v>
+        <v>0.19429399999999999</v>
       </c>
       <c r="I10" s="7">
-        <v>7.6900000000000004E-4</v>
+        <v>1.7030000000000001E-3</v>
       </c>
       <c r="J10" s="7">
-        <v>2.0760000000000002E-3</v>
+        <v>2.2160000000000001E-3</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -7290,26 +7617,26 @@
         <v>211874</v>
       </c>
       <c r="D11" s="7">
-        <v>64267</v>
+        <v>66527</v>
       </c>
       <c r="E11" s="14">
         <f t="shared" si="0"/>
-        <v>0.69667349462416339</v>
+        <v>0.68600677761310969</v>
       </c>
       <c r="F11" s="7">
         <v>3</v>
       </c>
       <c r="G11" s="7">
-        <v>12360</v>
+        <v>12703</v>
       </c>
       <c r="H11" s="7">
-        <v>7.9210000000000003E-2</v>
+        <v>9.9413000000000001E-2</v>
       </c>
       <c r="I11" s="7">
-        <v>1.06E-3</v>
+        <v>1.2149999999999999E-3</v>
       </c>
       <c r="J11" s="7">
-        <v>4.1900000000000001E-3</v>
+        <v>3.9370000000000004E-3</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -7323,26 +7650,26 @@
         <v>211874</v>
       </c>
       <c r="D12" s="7">
-        <v>44530</v>
+        <v>42555</v>
       </c>
       <c r="E12" s="14">
         <f t="shared" si="0"/>
-        <v>0.78982791659193674</v>
+        <v>0.79914949451088857</v>
       </c>
       <c r="F12" s="7">
         <v>3</v>
       </c>
       <c r="G12" s="7">
-        <v>4422</v>
+        <v>4149</v>
       </c>
       <c r="H12" s="7">
-        <v>5.8889999999999998E-2</v>
+        <v>5.5662999999999997E-2</v>
       </c>
       <c r="I12" s="7">
-        <v>1.2880000000000001E-3</v>
+        <v>1.299E-3</v>
       </c>
       <c r="J12" s="7">
-        <v>5.6230000000000004E-3</v>
+        <v>5.7930000000000004E-3</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -7356,11 +7683,11 @@
         <v>211874</v>
       </c>
       <c r="D13" s="7">
-        <v>34526</v>
+        <v>33178</v>
       </c>
       <c r="E13" s="14">
         <f t="shared" si="0"/>
-        <v>0.83704465861785782</v>
+        <v>0.84340693053418536</v>
       </c>
       <c r="F13" s="7">
         <v>2</v>
@@ -7372,10 +7699,10 @@
         <v>4.1445999999999997E-2</v>
       </c>
       <c r="I13" s="7">
-        <v>2.4120000000000001E-3</v>
+        <v>2.4269999999999999E-3</v>
       </c>
       <c r="J13" s="7">
-        <v>1.1686999999999999E-2</v>
+        <v>1.1776E-2</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -7389,11 +7716,11 @@
         <v>211874</v>
       </c>
       <c r="D14" s="7">
-        <v>21187</v>
+        <v>21172</v>
       </c>
       <c r="E14" s="14">
         <f t="shared" si="0"/>
-        <v>0.90000188791451519</v>
+        <v>0.90007268470883639</v>
       </c>
       <c r="F14" s="7">
         <v>1</v>
@@ -7405,10 +7732,10 @@
         <v>5.0117000000000002E-2</v>
       </c>
       <c r="I14" s="7">
-        <v>3.2079999999999999E-3</v>
+        <v>3.2160000000000001E-3</v>
       </c>
       <c r="J14" s="7">
-        <v>1.6726000000000001E-2</v>
+        <v>1.6778999999999999E-2</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -7422,26 +7749,26 @@
         <v>405680</v>
       </c>
       <c r="D15" s="7">
-        <v>118270</v>
+        <v>125308</v>
       </c>
       <c r="E15" s="14">
         <f t="shared" si="0"/>
-        <v>0.7084647998422402</v>
+        <v>0.69111615066061916</v>
       </c>
       <c r="F15" s="7">
         <v>3</v>
       </c>
       <c r="G15" s="7">
-        <v>8963</v>
+        <v>9795</v>
       </c>
       <c r="H15" s="7">
-        <v>0.11414000000000001</v>
+        <v>0.39617200000000002</v>
       </c>
       <c r="I15" s="7">
-        <v>1.0560000000000001E-3</v>
+        <v>3.6740000000000002E-3</v>
       </c>
       <c r="J15" s="7">
-        <v>3.8240000000000001E-3</v>
+        <v>4.6560000000000004E-3</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -7455,26 +7782,26 @@
         <v>405680</v>
       </c>
       <c r="D16" s="7">
-        <v>102499</v>
+        <v>106515</v>
       </c>
       <c r="E16" s="14">
         <f t="shared" si="0"/>
-        <v>0.74734026819167809</v>
+        <v>0.73744084007099198</v>
       </c>
       <c r="F16" s="7">
         <v>3</v>
       </c>
       <c r="G16" s="7">
-        <v>6031</v>
+        <v>5707</v>
       </c>
       <c r="H16" s="7">
-        <v>0.109976</v>
+        <v>0.35922599999999999</v>
       </c>
       <c r="I16" s="7">
-        <v>1.207E-3</v>
+        <v>3.2179999999999999E-3</v>
       </c>
       <c r="J16" s="7">
-        <v>4.2399999999999998E-3</v>
+        <v>4.9509999999999997E-3</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -7488,26 +7815,26 @@
         <v>405680</v>
       </c>
       <c r="D17" s="7">
-        <v>90425</v>
+        <v>98032</v>
       </c>
       <c r="E17" s="14">
         <f t="shared" si="0"/>
-        <v>0.77710264247682903</v>
+        <v>0.75835140997830797</v>
       </c>
       <c r="F17" s="7">
         <v>3</v>
       </c>
       <c r="G17" s="7">
-        <v>2808</v>
+        <v>4044</v>
       </c>
       <c r="H17" s="7">
-        <v>0.38563599999999998</v>
+        <v>0.36501400000000001</v>
       </c>
       <c r="I17" s="7">
-        <v>2.2239999999999998E-3</v>
+        <v>3.4250000000000001E-3</v>
       </c>
       <c r="J17" s="7">
-        <v>4.8209999999999998E-3</v>
+        <v>5.2230000000000002E-3</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -7521,11 +7848,11 @@
         <v>405680</v>
       </c>
       <c r="D18" s="7">
-        <v>40568</v>
+        <v>40563</v>
       </c>
       <c r="E18" s="14">
         <f t="shared" si="0"/>
-        <v>0.9</v>
+        <v>0.90001232498521</v>
       </c>
       <c r="F18" s="7">
         <v>1</v>
@@ -7540,7 +7867,7 @@
         <v>1.3680000000000001E-3</v>
       </c>
       <c r="J18" s="7">
-        <v>4.9020000000000001E-3</v>
+        <v>4.9030000000000002E-3</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -7554,11 +7881,11 @@
         <v>405680</v>
       </c>
       <c r="D19" s="7">
-        <v>40568</v>
+        <v>40563</v>
       </c>
       <c r="E19" s="14">
         <f t="shared" si="0"/>
-        <v>0.9</v>
+        <v>0.90001232498521</v>
       </c>
       <c r="F19" s="7">
         <v>1</v>
@@ -7573,7 +7900,7 @@
         <v>1.3680000000000001E-3</v>
       </c>
       <c r="J19" s="7">
-        <v>4.9020000000000001E-3</v>
+        <v>4.9030000000000002E-3</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -7752,11 +8079,11 @@
         <v>1869988</v>
       </c>
       <c r="D25" s="7">
-        <v>602117</v>
+        <v>575314</v>
       </c>
       <c r="E25" s="14">
         <f t="shared" si="0"/>
-        <v>0.67801023322074794</v>
+        <v>0.69234348027901782</v>
       </c>
       <c r="F25" s="7">
         <v>3</v>
@@ -7768,10 +8095,10 @@
         <v>1.2324E-2</v>
       </c>
       <c r="I25" s="7">
-        <v>1.462E-3</v>
+        <v>1.4779999999999999E-3</v>
       </c>
       <c r="J25" s="7">
-        <v>4.0309999999999999E-3</v>
+        <v>4.0359999999999997E-3</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -7785,11 +8112,11 @@
         <v>1869988</v>
       </c>
       <c r="D26" s="7">
-        <v>504414</v>
+        <v>478199</v>
       </c>
       <c r="E26" s="14">
         <f t="shared" si="0"/>
-        <v>0.73025816208446259</v>
+        <v>0.74427696862225856</v>
       </c>
       <c r="F26" s="7">
         <v>2</v>
@@ -7801,10 +8128,10 @@
         <v>1.1802E-2</v>
       </c>
       <c r="I26" s="7">
-        <v>1.8469999999999999E-3</v>
+        <v>1.867E-3</v>
       </c>
       <c r="J26" s="7">
-        <v>4.9300000000000004E-3</v>
+        <v>4.9439999999999996E-3</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
@@ -7927,12 +8254,12 @@
   <sheetData>
     <row r="1" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7940,7 +8267,7 @@
         <v>34</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>110</v>
@@ -7949,19 +8276,19 @@
         <v>111</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>143</v>
@@ -8012,11 +8339,11 @@
         <v>13790</v>
       </c>
       <c r="D6" s="7">
-        <v>6700</v>
+        <v>6484</v>
       </c>
       <c r="E6" s="14">
         <f t="shared" si="0"/>
-        <v>0.51414068165337201</v>
+        <v>0.52980420594633792</v>
       </c>
       <c r="F6" s="7">
         <v>12766</v>
@@ -8046,11 +8373,11 @@
         <v>13790</v>
       </c>
       <c r="D7" s="7">
-        <v>6644</v>
+        <v>6452</v>
       </c>
       <c r="E7" s="14">
         <f t="shared" si="0"/>
-        <v>0.51820159535895582</v>
+        <v>0.53212472806381439</v>
       </c>
       <c r="F7" s="7">
         <v>12042</v>
@@ -8080,24 +8407,24 @@
         <v>13790</v>
       </c>
       <c r="D8" s="7">
-        <v>5093</v>
+        <v>5231</v>
       </c>
       <c r="E8" s="14">
         <f t="shared" si="0"/>
-        <v>0.63067440174039158</v>
+        <v>0.62066715010877449</v>
       </c>
       <c r="F8" s="7">
-        <v>11279</v>
+        <v>11261</v>
       </c>
       <c r="G8" s="7">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="H8" s="14">
         <f t="shared" si="1"/>
-        <v>0.900079794308006</v>
+        <v>0.90000888020602077</v>
       </c>
       <c r="I8" s="7">
-        <v>6.9170000000000004E-3</v>
+        <v>7.9950000000000004E-3</v>
       </c>
       <c r="J8" s="7">
         <v>3</v>
@@ -8114,21 +8441,21 @@
         <v>13790</v>
       </c>
       <c r="D9" s="7">
-        <v>6698</v>
+        <v>6358</v>
       </c>
       <c r="E9" s="14">
         <f t="shared" si="0"/>
-        <v>0.51428571428571423</v>
+        <v>0.53894126178390134</v>
       </c>
       <c r="F9" s="7">
-        <v>9639</v>
+        <v>9834</v>
       </c>
       <c r="G9" s="7">
-        <v>481</v>
+        <v>491</v>
       </c>
       <c r="H9" s="14">
         <f t="shared" si="1"/>
-        <v>0.95009855794169518</v>
+        <v>0.95007118161480575</v>
       </c>
       <c r="I9" s="7">
         <v>2.3931999999999998E-2</v>
@@ -8216,11 +8543,11 @@
         <v>211874</v>
       </c>
       <c r="D12" s="7">
-        <v>42374</v>
+        <v>42372</v>
       </c>
       <c r="E12" s="14">
         <f t="shared" si="0"/>
-        <v>0.80000377582903048</v>
+        <v>0.80001321540160664</v>
       </c>
       <c r="F12" s="7">
         <v>211874</v>
@@ -8250,24 +8577,24 @@
         <v>211874</v>
       </c>
       <c r="D13" s="7">
-        <v>44530</v>
+        <v>42555</v>
       </c>
       <c r="E13" s="14">
         <f t="shared" si="0"/>
-        <v>0.78982791659193674</v>
+        <v>0.79914949451088857</v>
       </c>
       <c r="F13" s="7">
-        <v>201697</v>
+        <v>202363</v>
       </c>
       <c r="G13" s="7">
-        <v>20169</v>
+        <v>20236</v>
       </c>
       <c r="H13" s="14">
         <f t="shared" si="1"/>
-        <v>0.90000347055236318</v>
+        <v>0.90000148248444622</v>
       </c>
       <c r="I13" s="7">
-        <v>5.8889999999999998E-2</v>
+        <v>5.5662999999999997E-2</v>
       </c>
       <c r="J13" s="7">
         <v>3</v>
@@ -8284,24 +8611,24 @@
         <v>211874</v>
       </c>
       <c r="D14" s="7">
-        <v>35315</v>
+        <v>36457</v>
       </c>
       <c r="E14" s="14">
         <f t="shared" si="0"/>
-        <v>0.83332074723656513</v>
+        <v>0.82793075129558136</v>
       </c>
       <c r="F14" s="7">
-        <v>197445</v>
+        <v>196329</v>
       </c>
       <c r="G14" s="7">
-        <v>9872</v>
+        <v>9815</v>
       </c>
       <c r="H14" s="14">
         <f t="shared" si="1"/>
-        <v>0.9500012661753906</v>
+        <v>0.95000738556199038</v>
       </c>
       <c r="I14" s="7">
-        <v>0.166793</v>
+        <v>0.19270200000000001</v>
       </c>
       <c r="J14" s="7">
         <v>3</v>
@@ -8352,11 +8679,11 @@
         <v>405680</v>
       </c>
       <c r="D16" s="7">
-        <v>121704</v>
+        <v>121695</v>
       </c>
       <c r="E16" s="14">
         <f t="shared" si="0"/>
-        <v>0.7</v>
+        <v>0.70002218497337809</v>
       </c>
       <c r="F16" s="7">
         <v>405680</v>
@@ -8386,11 +8713,11 @@
         <v>405680</v>
       </c>
       <c r="D17" s="7">
-        <v>81136</v>
+        <v>81131</v>
       </c>
       <c r="E17" s="14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.80001232498521002</v>
       </c>
       <c r="F17" s="7">
         <v>405680</v>
@@ -8420,24 +8747,24 @@
         <v>405680</v>
       </c>
       <c r="D18" s="7">
-        <v>90425</v>
+        <v>98032</v>
       </c>
       <c r="E18" s="14">
         <f t="shared" si="0"/>
-        <v>0.77710264247682903</v>
+        <v>0.75835140997830797</v>
       </c>
       <c r="F18" s="7">
-        <v>395213</v>
+        <v>390925</v>
       </c>
       <c r="G18" s="7">
-        <v>39521</v>
+        <v>39092</v>
       </c>
       <c r="H18" s="14">
         <f t="shared" si="1"/>
-        <v>0.90000075908434185</v>
+        <v>0.90000127901771443</v>
       </c>
       <c r="I18" s="7">
-        <v>0.38563599999999998</v>
+        <v>0.36501400000000001</v>
       </c>
       <c r="J18" s="7">
         <v>3</v>
@@ -8454,24 +8781,24 @@
         <v>405680</v>
       </c>
       <c r="D19" s="7">
-        <v>51200</v>
+        <v>48046</v>
       </c>
       <c r="E19" s="14">
         <f t="shared" si="0"/>
-        <v>0.87379215144941824</v>
+        <v>0.88156675211989743</v>
       </c>
       <c r="F19" s="7">
-        <v>400258</v>
+        <v>401031</v>
       </c>
       <c r="G19" s="7">
-        <v>20012</v>
+        <v>20051</v>
       </c>
       <c r="H19" s="14">
         <f t="shared" si="1"/>
-        <v>0.9500022485496854</v>
+        <v>0.95000137146504882</v>
       </c>
       <c r="I19" s="7">
-        <v>0.19997000000000001</v>
+        <v>0.31517000000000001</v>
       </c>
       <c r="J19" s="7">
         <v>3</v>
@@ -8794,11 +9121,11 @@
         <v>1869988</v>
       </c>
       <c r="D29" s="7">
-        <v>281484</v>
+        <v>265646</v>
       </c>
       <c r="E29" s="14">
         <f t="shared" si="0"/>
-        <v>0.84947283084169523</v>
+        <v>0.85794240390847432</v>
       </c>
       <c r="F29" s="7">
         <v>1869984</v>
@@ -8841,12 +9168,12 @@
   <sheetData>
     <row r="1" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -8854,10 +9181,10 @@
         <v>34</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>110</v>
@@ -8866,13 +9193,13 @@
         <v>111</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>144</v>
@@ -8881,10 +9208,10 @@
         <v>143</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -8892,7 +9219,7 @@
         <v>45</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C5" s="7">
         <v>90</v>
@@ -8931,7 +9258,7 @@
         <v>45</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C6" s="7">
         <v>90</v>
@@ -8970,7 +9297,7 @@
         <v>52</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C7" s="7">
         <v>90</v>
@@ -9009,7 +9336,7 @@
         <v>52</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C8" s="7">
         <v>90</v>
@@ -9048,7 +9375,7 @@
         <v>55</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C9" s="7">
         <v>90</v>
@@ -9087,7 +9414,7 @@
         <v>55</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C10" s="7">
         <v>90</v>
@@ -9126,7 +9453,7 @@
         <v>58</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C11" s="7">
         <v>90</v>
@@ -9165,7 +9492,7 @@
         <v>58</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C12" s="7">
         <v>90</v>
@@ -9204,7 +9531,7 @@
         <v>62</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C13" s="7">
         <v>90</v>
@@ -9243,7 +9570,7 @@
         <v>62</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C14" s="7">
         <v>90</v>
@@ -9282,7 +9609,7 @@
         <v>64</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C15" s="7">
         <v>90</v>
@@ -9321,7 +9648,7 @@
         <v>64</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C16" s="7">
         <v>90</v>
@@ -9360,7 +9687,7 @@
         <v>66</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C17" s="7">
         <v>90</v>
@@ -9399,7 +9726,7 @@
         <v>66</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C18" s="7">
         <v>90</v>
@@ -9438,7 +9765,7 @@
         <v>69</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C19" s="7">
         <v>90</v>
@@ -9477,7 +9804,7 @@
         <v>69</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C20" s="7">
         <v>90</v>
@@ -9516,7 +9843,7 @@
         <v>71</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C21" s="7">
         <v>90</v>
@@ -9555,7 +9882,7 @@
         <v>71</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C22" s="7">
         <v>90</v>
@@ -9594,7 +9921,7 @@
         <v>75</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C23" s="7">
         <v>90</v>
@@ -9633,7 +9960,7 @@
         <v>75</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C24" s="7">
         <v>90</v>
@@ -9672,7 +9999,7 @@
         <v>78</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C25" s="7">
         <v>90</v>
@@ -9711,7 +10038,7 @@
         <v>78</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C26" s="7">
         <v>90</v>
@@ -9750,7 +10077,7 @@
         <v>80</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C27" s="7">
         <v>90</v>
@@ -9789,7 +10116,7 @@
         <v>80</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C28" s="7">
         <v>90</v>
@@ -9828,7 +10155,7 @@
         <v>83</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C29" s="7">
         <v>90</v>
@@ -9867,7 +10194,7 @@
         <v>83</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C30" s="7">
         <v>90</v>
@@ -9906,7 +10233,7 @@
         <v>88</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C31" s="7">
         <v>90</v>
@@ -9945,7 +10272,7 @@
         <v>88</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C32" s="7">
         <v>90</v>
@@ -9984,7 +10311,7 @@
         <v>90</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C33" s="7">
         <v>90</v>
@@ -10023,7 +10350,7 @@
         <v>90</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C34" s="7">
         <v>90</v>
@@ -10062,7 +10389,7 @@
         <v>93</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C35" s="7">
         <v>90</v>
@@ -10101,7 +10428,7 @@
         <v>93</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C36" s="7">
         <v>90</v>
@@ -10140,7 +10467,7 @@
         <v>97</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C37" s="7">
         <v>90</v>
@@ -10179,7 +10506,7 @@
         <v>97</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C38" s="7">
         <v>90</v>
@@ -10218,7 +10545,7 @@
         <v>99</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C39" s="7">
         <v>90</v>
@@ -10257,7 +10584,7 @@
         <v>99</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C40" s="7">
         <v>90</v>
@@ -10296,7 +10623,7 @@
         <v>104</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C41" s="7">
         <v>90</v>
@@ -10335,7 +10662,7 @@
         <v>104</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C42" s="7">
         <v>90</v>
@@ -10388,12 +10715,12 @@
   <sheetData>
     <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -10401,30 +10728,30 @@
         <v>34</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B5" s="7">
         <v>0</v>
@@ -10441,18 +10768,18 @@
         <v/>
       </c>
       <c r="F5" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B6" s="7">
         <v>0</v>
@@ -10469,18 +10796,18 @@
         <v/>
       </c>
       <c r="F6" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B7" s="7">
         <v>12</v>
@@ -10497,18 +10824,18 @@
         <v>1</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B8" s="7">
         <v>12</v>
@@ -10525,18 +10852,18 @@
         <v>1</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B9" s="7">
         <v>20</v>
@@ -10553,18 +10880,18 @@
         <v>1</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B10" s="7">
         <v>20</v>
@@ -10581,18 +10908,18 @@
         <v>1</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B11" s="7">
         <v>32</v>
@@ -10609,18 +10936,18 @@
         <v>1</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B12" s="7">
         <v>32</v>
@@ -10637,18 +10964,18 @@
         <v>1</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B13" s="7">
         <v>32</v>
@@ -10665,18 +10992,18 @@
         <v>1</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B14" s="7">
         <v>32</v>
@@ -10693,18 +11020,18 @@
         <v>1</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B15" s="7">
         <v>40</v>
@@ -10721,18 +11048,18 @@
         <v>1</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B16" s="7">
         <v>40</v>
@@ -10749,13 +11076,13 @@
         <v>1</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fix seam repair for open-boundary meshes
Preserve real source openings during protected-zone decimation by tracking source boundary vertices and skipping seam caps on genuine mesh holes. refine_by_error now keeps the best pass instead of always accepting later refinements, and adds regression tests covering open-boundary and non-worsening behavior. This also adds the baseline comparison experiment script and refreshed evaluation result artifacts under evaluation/results.
</commit_message>
<xml_diff>
--- a/evaluation/evaluation_tracker.xlsx
+++ b/evaluation/evaluation_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnniDin00\Documents\GitHub\adaptive-remesher\evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C80CE13C-11F8-4713-961A-EF29D8D5BD72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24C23491-2475-4750-87B7-6C2E553C19B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,6 +24,7 @@
     <sheet name="UV_Seam_Detection" sheetId="9" r:id="rId9"/>
     <sheet name="Validity_Checks" sheetId="10" r:id="rId10"/>
     <sheet name="Runtime" sheetId="11" r:id="rId11"/>
+    <sheet name="Baselines" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="793" uniqueCount="248">
   <si>
     <t>Adaptive Remesher — Evaluation Data Tracker</t>
   </si>
@@ -751,6 +752,42 @@
   </si>
   <si>
     <t>Default pipeline (DecimatePro, 90%, UV+auto-error protection)</t>
+  </si>
+  <si>
+    <t>Baseline comparison (fixed 90% reduction): E_max pooled as % of bbox diagonal</t>
+  </si>
+  <si>
+    <t>Adaptive Remesher = Experiment B (unprotected 90% / refined); MeshLab QEM = PyMeshLab quadric edge collapse, defaults; fast-simplification = Python quadric simplifier. All scored with the same bidirectional measure.</t>
+  </si>
+  <si>
+    <t>AR no refinement (%)</t>
+  </si>
+  <si>
+    <t>AR refined (%)</t>
+  </si>
+  <si>
+    <t>AR refined reduction (%)</t>
+  </si>
+  <si>
+    <t>MeshLab QEM (%)</t>
+  </si>
+  <si>
+    <t>MeshLab QEM boundary (%)</t>
+  </si>
+  <si>
+    <t>MeshLab QEM boundary reduction achieved (%)</t>
+  </si>
+  <si>
+    <t>fast-simplification (%)</t>
+  </si>
+  <si>
+    <t>Median</t>
+  </si>
+  <si>
+    <t>Mean</t>
+  </si>
+  <si>
+    <t>Note: MeshLab with boundary preservation fails to reduce some meshes (see column I) and produced a degenerate result on Bolt Cutters; it is excluded from the medians.</t>
   </si>
 </sst>
 </file>
@@ -761,7 +798,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -821,6 +858,11 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -872,7 +914,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -904,6 +946,7 @@
     <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
@@ -1663,7 +1706,7 @@
         <v>227</v>
       </c>
       <c r="C12" s="7">
-        <v>1386</v>
+        <v>1369</v>
       </c>
       <c r="D12" s="7">
         <v>697</v>
@@ -1672,7 +1715,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="7">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="G12" s="7">
         <v>0</v>
@@ -1685,7 +1728,7 @@
       </c>
       <c r="J12" s="15" t="str">
         <f t="shared" si="0"/>
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -1861,16 +1904,16 @@
         <v>227</v>
       </c>
       <c r="C18" s="7">
-        <v>3192</v>
+        <v>2928</v>
       </c>
       <c r="D18" s="7">
-        <v>1642</v>
+        <v>1621</v>
       </c>
       <c r="E18" s="7">
         <v>0</v>
       </c>
       <c r="F18" s="7">
-        <v>0</v>
+        <v>264</v>
       </c>
       <c r="G18" s="7">
         <v>0</v>
@@ -1883,7 +1926,7 @@
       </c>
       <c r="J18" s="15" t="str">
         <f t="shared" si="0"/>
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -1927,29 +1970,29 @@
         <v>227</v>
       </c>
       <c r="C20" s="7">
-        <v>2642</v>
+        <v>2302</v>
       </c>
       <c r="D20" s="7">
-        <v>1365</v>
+        <v>1350</v>
       </c>
       <c r="E20" s="7">
         <v>0</v>
       </c>
       <c r="F20" s="7">
-        <v>0</v>
+        <v>362</v>
       </c>
       <c r="G20" s="7">
         <v>0</v>
       </c>
       <c r="H20" s="7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I20" s="7">
         <v>22</v>
       </c>
       <c r="J20" s="15" t="str">
         <f t="shared" si="0"/>
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -2455,16 +2498,16 @@
         <v>227</v>
       </c>
       <c r="C36" s="7">
-        <v>8112</v>
+        <v>7769</v>
       </c>
       <c r="D36" s="7">
-        <v>4059</v>
+        <v>3994</v>
       </c>
       <c r="E36" s="7">
         <v>0</v>
       </c>
       <c r="F36" s="7">
-        <v>0</v>
+        <v>223</v>
       </c>
       <c r="G36" s="7">
         <v>0</v>
@@ -2477,7 +2520,7 @@
       </c>
       <c r="J36" s="15" t="str">
         <f t="shared" si="0"/>
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
@@ -2744,16 +2787,16 @@
         <v>235</v>
       </c>
       <c r="D5" s="7">
-        <v>0.45650000000000002</v>
+        <v>0.48899999999999999</v>
       </c>
       <c r="E5" s="7">
-        <v>0.19420000000000001</v>
+        <v>0.20469999999999999</v>
       </c>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
       <c r="H5" s="15">
         <f t="shared" ref="H5:H29" si="0">IFERROR(D5-SUM(E5:G5),"")</f>
-        <v>0.26229999999999998</v>
+        <v>0.2843</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -2767,16 +2810,16 @@
         <v>235</v>
       </c>
       <c r="D6" s="7">
-        <v>0.1956</v>
+        <v>0.20300000000000001</v>
       </c>
       <c r="E6" s="7">
-        <v>4.7E-2</v>
+        <v>4.8500000000000001E-2</v>
       </c>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
       <c r="H6" s="15">
         <f t="shared" si="0"/>
-        <v>0.14860000000000001</v>
+        <v>0.15450000000000003</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -2790,16 +2833,16 @@
         <v>235</v>
       </c>
       <c r="D7" s="7">
-        <v>0.92090000000000005</v>
+        <v>0.98129999999999995</v>
       </c>
       <c r="E7" s="7">
-        <v>0.38979999999999998</v>
+        <v>0.41620000000000001</v>
       </c>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
       <c r="H7" s="15">
         <f t="shared" si="0"/>
-        <v>0.53110000000000013</v>
+        <v>0.56509999999999994</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -2813,16 +2856,16 @@
         <v>235</v>
       </c>
       <c r="D8" s="7">
-        <v>1.9400000000000001E-2</v>
+        <v>2.0199999999999999E-2</v>
       </c>
       <c r="E8" s="7">
-        <v>9.9000000000000008E-3</v>
+        <v>0.01</v>
       </c>
       <c r="F8" s="7"/>
       <c r="G8" s="7"/>
       <c r="H8" s="15">
         <f t="shared" si="0"/>
-        <v>9.4999999999999998E-3</v>
+        <v>1.0199999999999999E-2</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -2836,16 +2879,16 @@
         <v>235</v>
       </c>
       <c r="D9" s="7">
-        <v>0.2646</v>
+        <v>0.2707</v>
       </c>
       <c r="E9" s="7">
-        <v>3.7400000000000003E-2</v>
+        <v>3.9E-2</v>
       </c>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
       <c r="H9" s="15">
         <f t="shared" si="0"/>
-        <v>0.22720000000000001</v>
+        <v>0.23169999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -2859,16 +2902,16 @@
         <v>235</v>
       </c>
       <c r="D10" s="7">
-        <v>5.3800000000000001E-2</v>
+        <v>5.2499999999999998E-2</v>
       </c>
       <c r="E10" s="7">
-        <v>1.43E-2</v>
+        <v>1.3299999999999999E-2</v>
       </c>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
       <c r="H10" s="15">
         <f t="shared" si="0"/>
-        <v>3.95E-2</v>
+        <v>3.9199999999999999E-2</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -2882,16 +2925,16 @@
         <v>235</v>
       </c>
       <c r="D11" s="7">
-        <v>4.1000000000000002E-2</v>
+        <v>3.7900000000000003E-2</v>
       </c>
       <c r="E11" s="7">
-        <v>1.9800000000000002E-2</v>
+        <v>1.7399999999999999E-2</v>
       </c>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
       <c r="H11" s="15">
         <f t="shared" si="0"/>
-        <v>2.12E-2</v>
+        <v>2.0500000000000004E-2</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -2905,16 +2948,16 @@
         <v>235</v>
       </c>
       <c r="D12" s="7">
-        <v>9.3600000000000003E-2</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="E12" s="7">
-        <v>1.6400000000000001E-2</v>
+        <v>2.0799999999999999E-2</v>
       </c>
       <c r="F12" s="7"/>
       <c r="G12" s="7"/>
       <c r="H12" s="15">
         <f t="shared" si="0"/>
-        <v>7.7200000000000005E-2</v>
+        <v>2.0200000000000003E-2</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -2928,16 +2971,16 @@
         <v>235</v>
       </c>
       <c r="D13" s="7">
-        <v>1.5322</v>
+        <v>1.8729</v>
       </c>
       <c r="E13" s="7">
-        <v>0.72789999999999999</v>
+        <v>0.97360000000000002</v>
       </c>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
       <c r="H13" s="15">
         <f t="shared" si="0"/>
-        <v>0.80430000000000001</v>
+        <v>0.89929999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -2951,16 +2994,16 @@
         <v>235</v>
       </c>
       <c r="D14" s="7">
-        <v>3.7456</v>
+        <v>4.3567</v>
       </c>
       <c r="E14" s="7">
-        <v>1.7293000000000001</v>
+        <v>2.0836999999999999</v>
       </c>
       <c r="F14" s="7"/>
       <c r="G14" s="7"/>
       <c r="H14" s="15">
         <f t="shared" si="0"/>
-        <v>2.0163000000000002</v>
+        <v>2.2730000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -2974,16 +3017,16 @@
         <v>235</v>
       </c>
       <c r="D15" s="7">
-        <v>0.91800000000000004</v>
+        <v>1.0666</v>
       </c>
       <c r="E15" s="7">
-        <v>0.36420000000000002</v>
+        <v>0.43990000000000001</v>
       </c>
       <c r="F15" s="7"/>
       <c r="G15" s="7"/>
       <c r="H15" s="15">
         <f t="shared" si="0"/>
-        <v>0.55380000000000007</v>
+        <v>0.62670000000000003</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -2997,16 +3040,16 @@
         <v>235</v>
       </c>
       <c r="D16" s="7">
-        <v>4.5187999999999997</v>
+        <v>4.8358999999999996</v>
       </c>
       <c r="E16" s="7">
-        <v>1.1801999999999999</v>
+        <v>1.4262999999999999</v>
       </c>
       <c r="F16" s="7"/>
       <c r="G16" s="7"/>
       <c r="H16" s="15">
         <f t="shared" si="0"/>
-        <v>3.3385999999999996</v>
+        <v>3.4095999999999997</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -3020,16 +3063,16 @@
         <v>235</v>
       </c>
       <c r="D17" s="7">
-        <v>0.12820000000000001</v>
+        <v>0.12920000000000001</v>
       </c>
       <c r="E17" s="7">
-        <v>2.9700000000000001E-2</v>
+        <v>2.8400000000000002E-2</v>
       </c>
       <c r="F17" s="7"/>
       <c r="G17" s="7"/>
       <c r="H17" s="15">
         <f t="shared" si="0"/>
-        <v>9.8500000000000004E-2</v>
+        <v>0.1008</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -3043,16 +3086,16 @@
         <v>235</v>
       </c>
       <c r="D18" s="7">
-        <v>0.18909999999999999</v>
+        <v>0.2044</v>
       </c>
       <c r="E18" s="7">
-        <v>5.8500000000000003E-2</v>
+        <v>6.3600000000000004E-2</v>
       </c>
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
       <c r="H18" s="15">
         <f t="shared" si="0"/>
-        <v>0.13059999999999999</v>
+        <v>0.14079999999999998</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -3066,16 +3109,16 @@
         <v>235</v>
       </c>
       <c r="D19" s="7">
-        <v>0.46</v>
+        <v>0.52159999999999995</v>
       </c>
       <c r="E19" s="7">
-        <v>0.19950000000000001</v>
+        <v>0.22889999999999999</v>
       </c>
       <c r="F19" s="7"/>
       <c r="G19" s="7"/>
       <c r="H19" s="15">
         <f t="shared" si="0"/>
-        <v>0.26050000000000001</v>
+        <v>0.29269999999999996</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -3089,16 +3132,16 @@
         <v>235</v>
       </c>
       <c r="D20" s="7">
-        <v>1.1100000000000001</v>
+        <v>0.77639999999999998</v>
       </c>
       <c r="E20" s="7">
-        <v>0.19270000000000001</v>
+        <v>0.20169999999999999</v>
       </c>
       <c r="F20" s="7"/>
       <c r="G20" s="7"/>
       <c r="H20" s="15">
         <f t="shared" si="0"/>
-        <v>0.91730000000000012</v>
+        <v>0.57469999999999999</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -3112,16 +3155,16 @@
         <v>235</v>
       </c>
       <c r="D21" s="7">
-        <v>2.7427999999999999</v>
+        <v>3.3696000000000002</v>
       </c>
       <c r="E21" s="7">
-        <v>1.5616000000000001</v>
+        <v>1.9644999999999999</v>
       </c>
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
       <c r="H21" s="15">
         <f t="shared" si="0"/>
-        <v>1.1811999999999998</v>
+        <v>1.4051000000000002</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -3135,16 +3178,16 @@
         <v>235</v>
       </c>
       <c r="D22" s="7">
-        <v>33.584800000000001</v>
+        <v>32.713299999999997</v>
       </c>
       <c r="E22" s="7">
-        <v>12.879300000000001</v>
+        <v>13.2342</v>
       </c>
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
       <c r="H22" s="15">
         <f t="shared" si="0"/>
-        <v>20.705500000000001</v>
+        <v>19.479099999999995</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -3158,16 +3201,16 @@
         <v>235</v>
       </c>
       <c r="D23" s="7">
-        <v>1.0643</v>
+        <v>1.1264000000000001</v>
       </c>
       <c r="E23" s="7">
-        <v>0.1172</v>
+        <v>0.13039999999999999</v>
       </c>
       <c r="F23" s="7"/>
       <c r="G23" s="7"/>
       <c r="H23" s="15">
         <f t="shared" si="0"/>
-        <v>0.94710000000000005</v>
+        <v>0.99600000000000011</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -3246,6 +3289,717 @@
       <c r="H29" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
+  <dimension ref="A1:J28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="2" max="10" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="21" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>238</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>239</v>
+      </c>
+      <c r="F4" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="G4" s="21" t="s">
+        <v>241</v>
+      </c>
+      <c r="H4" s="21" t="s">
+        <v>242</v>
+      </c>
+      <c r="I4" s="21" t="s">
+        <v>243</v>
+      </c>
+      <c r="J4" s="21" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5">
+        <v>59996</v>
+      </c>
+      <c r="D5">
+        <v>0.45050000000000001</v>
+      </c>
+      <c r="E5">
+        <v>0.45050000000000001</v>
+      </c>
+      <c r="F5">
+        <v>90</v>
+      </c>
+      <c r="G5">
+        <v>0.84219999999999995</v>
+      </c>
+      <c r="H5">
+        <v>0.78620000000000001</v>
+      </c>
+      <c r="I5">
+        <v>90</v>
+      </c>
+      <c r="J5">
+        <v>0.81969999999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6">
+        <v>15000</v>
+      </c>
+      <c r="D6">
+        <v>0.45469999999999999</v>
+      </c>
+      <c r="E6">
+        <v>0.45469999999999999</v>
+      </c>
+      <c r="F6">
+        <v>90</v>
+      </c>
+      <c r="G6">
+        <v>0.4627</v>
+      </c>
+      <c r="H6">
+        <v>0.5978</v>
+      </c>
+      <c r="I6">
+        <v>90</v>
+      </c>
+      <c r="J6">
+        <v>0.69710000000000005</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7">
+        <v>130504</v>
+      </c>
+      <c r="D7">
+        <v>0.23</v>
+      </c>
+      <c r="E7">
+        <v>0.23</v>
+      </c>
+      <c r="F7">
+        <v>90</v>
+      </c>
+      <c r="G7">
+        <v>0.25779999999999997</v>
+      </c>
+      <c r="H7">
+        <v>0.26979999999999998</v>
+      </c>
+      <c r="I7">
+        <v>90</v>
+      </c>
+      <c r="J7">
+        <v>0.77349999999999997</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8">
+        <v>1473</v>
+      </c>
+      <c r="D8">
+        <v>611.51469999999995</v>
+      </c>
+      <c r="E8">
+        <v>3.8822999999999999</v>
+      </c>
+      <c r="F8">
+        <v>2.17</v>
+      </c>
+      <c r="G8">
+        <v>2.8645999999999998</v>
+      </c>
+      <c r="H8">
+        <v>8.4971999999999994</v>
+      </c>
+      <c r="I8">
+        <v>50.1</v>
+      </c>
+      <c r="J8">
+        <v>16.055299999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9">
+        <v>13790</v>
+      </c>
+      <c r="D9">
+        <v>6.2081999999999997</v>
+      </c>
+      <c r="E9">
+        <v>2.3178999999999998</v>
+      </c>
+      <c r="F9">
+        <v>62.76</v>
+      </c>
+      <c r="G9">
+        <v>3.4849999999999999</v>
+      </c>
+      <c r="H9">
+        <v>5.0763999999999996</v>
+      </c>
+      <c r="I9">
+        <v>69.37</v>
+      </c>
+      <c r="J9">
+        <v>4.9196999999999997</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10">
+        <v>2752</v>
+      </c>
+      <c r="D10">
+        <v>6.5776000000000003</v>
+      </c>
+      <c r="E10">
+        <v>1.2259</v>
+      </c>
+      <c r="F10">
+        <v>-1.38</v>
+      </c>
+      <c r="G10">
+        <v>6.1483999999999996</v>
+      </c>
+      <c r="H10">
+        <v>7.9634</v>
+      </c>
+      <c r="I10">
+        <v>79.58</v>
+      </c>
+      <c r="J10">
+        <v>4.2689000000000004</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11">
+        <v>3410</v>
+      </c>
+      <c r="D11">
+        <v>14.7905</v>
+      </c>
+      <c r="E11">
+        <v>0.83979999999999999</v>
+      </c>
+      <c r="F11">
+        <v>70.260000000000005</v>
+      </c>
+      <c r="G11">
+        <v>1.2423999999999999</v>
+      </c>
+      <c r="H11">
+        <v>57055.814100000003</v>
+      </c>
+      <c r="I11">
+        <v>67.8</v>
+      </c>
+      <c r="J11">
+        <v>1.6878</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12">
+        <v>2926</v>
+      </c>
+      <c r="D12">
+        <v>17.108499999999999</v>
+      </c>
+      <c r="E12">
+        <v>3.6714000000000002</v>
+      </c>
+      <c r="F12">
+        <v>25.19</v>
+      </c>
+      <c r="G12">
+        <v>5.8425000000000002</v>
+      </c>
+      <c r="H12">
+        <v>3.2086000000000001</v>
+      </c>
+      <c r="I12">
+        <v>53.25</v>
+      </c>
+      <c r="J12">
+        <v>5.7952000000000004</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13">
+        <v>211874</v>
+      </c>
+      <c r="D13">
+        <v>2.1846000000000001</v>
+      </c>
+      <c r="E13">
+        <v>2.1846000000000001</v>
+      </c>
+      <c r="F13">
+        <v>90.01</v>
+      </c>
+      <c r="G13">
+        <v>1.9409000000000001</v>
+      </c>
+      <c r="H13">
+        <v>8.3651</v>
+      </c>
+      <c r="I13">
+        <v>85.2</v>
+      </c>
+      <c r="J13">
+        <v>1.3089</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" t="s">
+        <v>72</v>
+      </c>
+      <c r="C14">
+        <v>446670</v>
+      </c>
+      <c r="D14">
+        <v>1.9573</v>
+      </c>
+      <c r="E14">
+        <v>1.9573</v>
+      </c>
+      <c r="F14">
+        <v>90.01</v>
+      </c>
+      <c r="G14">
+        <v>3.6808999999999998</v>
+      </c>
+      <c r="H14">
+        <v>4.2846000000000002</v>
+      </c>
+      <c r="I14">
+        <v>74.819999999999993</v>
+      </c>
+      <c r="J14">
+        <v>0.65739999999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C15">
+        <v>108958</v>
+      </c>
+      <c r="D15">
+        <v>0.23419999999999999</v>
+      </c>
+      <c r="E15">
+        <v>0.23419999999999999</v>
+      </c>
+      <c r="F15">
+        <v>90.01</v>
+      </c>
+      <c r="G15">
+        <v>2.2921999999999998</v>
+      </c>
+      <c r="H15">
+        <v>0.14610000000000001</v>
+      </c>
+      <c r="I15">
+        <v>90</v>
+      </c>
+      <c r="J15">
+        <v>1.7793000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>80</v>
+      </c>
+      <c r="B16" t="s">
+        <v>72</v>
+      </c>
+      <c r="C16">
+        <v>405680</v>
+      </c>
+      <c r="D16">
+        <v>1.0354000000000001</v>
+      </c>
+      <c r="E16">
+        <v>1.0354000000000001</v>
+      </c>
+      <c r="F16">
+        <v>90</v>
+      </c>
+      <c r="G16">
+        <v>1.2028000000000001</v>
+      </c>
+      <c r="H16">
+        <v>1.1989000000000001</v>
+      </c>
+      <c r="I16">
+        <v>65.64</v>
+      </c>
+      <c r="J16">
+        <v>0.83030000000000004</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>83</v>
+      </c>
+      <c r="B17" t="s">
+        <v>84</v>
+      </c>
+      <c r="C17">
+        <v>5912</v>
+      </c>
+      <c r="D17">
+        <v>8.7843</v>
+      </c>
+      <c r="E17">
+        <v>3.4725999999999999</v>
+      </c>
+      <c r="F17">
+        <v>22.55</v>
+      </c>
+      <c r="G17">
+        <v>5.9821</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>11.137600000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>88</v>
+      </c>
+      <c r="B18" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18">
+        <v>16694</v>
+      </c>
+      <c r="D18">
+        <v>7.1600999999999999</v>
+      </c>
+      <c r="E18">
+        <v>1.996</v>
+      </c>
+      <c r="F18">
+        <v>29.27</v>
+      </c>
+      <c r="G18">
+        <v>7.0003000000000002</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>10.388</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>90</v>
+      </c>
+      <c r="B19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C19">
+        <v>63998</v>
+      </c>
+      <c r="D19">
+        <v>1.1271</v>
+      </c>
+      <c r="E19">
+        <v>0.92700000000000005</v>
+      </c>
+      <c r="F19">
+        <v>89.8</v>
+      </c>
+      <c r="G19">
+        <v>0.6865</v>
+      </c>
+      <c r="H19">
+        <v>1.0316000000000001</v>
+      </c>
+      <c r="I19">
+        <v>90</v>
+      </c>
+      <c r="J19">
+        <v>0.9083</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" t="s">
+        <v>84</v>
+      </c>
+      <c r="C20">
+        <v>69451</v>
+      </c>
+      <c r="D20">
+        <v>0.16700000000000001</v>
+      </c>
+      <c r="E20">
+        <v>0.16700000000000001</v>
+      </c>
+      <c r="F20">
+        <v>90</v>
+      </c>
+      <c r="G20">
+        <v>0.15210000000000001</v>
+      </c>
+      <c r="H20">
+        <v>0.18920000000000001</v>
+      </c>
+      <c r="I20">
+        <v>90</v>
+      </c>
+      <c r="J20">
+        <v>0.88109999999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>97</v>
+      </c>
+      <c r="B21" t="s">
+        <v>84</v>
+      </c>
+      <c r="C21">
+        <v>345944</v>
+      </c>
+      <c r="D21">
+        <v>7.6499999999999999E-2</v>
+      </c>
+      <c r="E21">
+        <v>7.6499999999999999E-2</v>
+      </c>
+      <c r="F21">
+        <v>90</v>
+      </c>
+      <c r="G21">
+        <v>8.7499999999999994E-2</v>
+      </c>
+      <c r="H21">
+        <v>8.7499999999999994E-2</v>
+      </c>
+      <c r="I21">
+        <v>90</v>
+      </c>
+      <c r="J21">
+        <v>7.8399999999999997E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>99</v>
+      </c>
+      <c r="B22" t="s">
+        <v>100</v>
+      </c>
+      <c r="C22">
+        <v>1869988</v>
+      </c>
+      <c r="D22">
+        <v>0.7964</v>
+      </c>
+      <c r="E22">
+        <v>0.7964</v>
+      </c>
+      <c r="F22">
+        <v>90</v>
+      </c>
+      <c r="G22">
+        <v>0.78420000000000001</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>2.5036</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>104</v>
+      </c>
+      <c r="B23" t="s">
+        <v>100</v>
+      </c>
+      <c r="C23">
+        <v>31400</v>
+      </c>
+      <c r="D23">
+        <v>5.2518000000000002</v>
+      </c>
+      <c r="E23">
+        <v>5.0335000000000001</v>
+      </c>
+      <c r="F23">
+        <v>27.93</v>
+      </c>
+      <c r="G23">
+        <v>7.6422999999999996</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>5.2385999999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="21" t="s">
+        <v>245</v>
+      </c>
+      <c r="D25">
+        <f>MEDIAN(D5:D23)</f>
+        <v>1.9573</v>
+      </c>
+      <c r="E25">
+        <f>MEDIAN(E5:E23)</f>
+        <v>1.0354000000000001</v>
+      </c>
+      <c r="G25">
+        <f>MEDIAN(G5:G23)</f>
+        <v>1.9409000000000001</v>
+      </c>
+      <c r="J25">
+        <f>MEDIAN(J5:J23)</f>
+        <v>1.6878</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="21" t="s">
+        <v>246</v>
+      </c>
+      <c r="D26">
+        <f>AVERAGE(D5:D23)</f>
+        <v>36.111021052631585</v>
+      </c>
+      <c r="E26">
+        <f>AVERAGE(E5:E23)</f>
+        <v>1.6291052631578946</v>
+      </c>
+      <c r="G26">
+        <f>AVERAGE(G5:G23)</f>
+        <v>2.7682842105263159</v>
+      </c>
+      <c r="J26">
+        <f>AVERAGE(J5:J23)</f>
+        <v>3.7225631578947369</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -4244,23 +4998,23 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="22"/>
-      <c r="M10" s="22"/>
-      <c r="N10" s="22"/>
-      <c r="O10" s="22"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="23"/>
+      <c r="O10" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4421,7 +5175,7 @@
         <v>0</v>
       </c>
       <c r="Q6" s="7">
-        <v>0.72799999999999998</v>
+        <v>0.84799999999999998</v>
       </c>
       <c r="R6" s="15" t="str">
         <f t="shared" ref="R6:R43" si="2">IFERROR(IF(M6/S6&gt;$D$3,"Yes","No"),"")</f>
@@ -4488,7 +5242,7 @@
         <v>1</v>
       </c>
       <c r="Q7" s="7">
-        <v>0.161</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="R7" s="15" t="str">
         <f t="shared" si="2"/>
@@ -4555,7 +5309,7 @@
         <v>0</v>
       </c>
       <c r="Q8" s="7">
-        <v>0.14099999999999999</v>
+        <v>0.17100000000000001</v>
       </c>
       <c r="R8" s="15" t="str">
         <f t="shared" si="2"/>
@@ -4622,7 +5376,7 @@
         <v>1</v>
       </c>
       <c r="Q9" s="7">
-        <v>3.7999999999999999E-2</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="R9" s="15" t="str">
         <f t="shared" si="2"/>
@@ -4689,7 +5443,7 @@
         <v>0</v>
       </c>
       <c r="Q10" s="7">
-        <v>1.4219999999999999</v>
+        <v>1.6990000000000001</v>
       </c>
       <c r="R10" s="15" t="str">
         <f t="shared" si="2"/>
@@ -4756,7 +5510,7 @@
         <v>1</v>
       </c>
       <c r="Q11" s="7">
-        <v>0.33200000000000002</v>
+        <v>0.48</v>
       </c>
       <c r="R11" s="15" t="str">
         <f t="shared" si="2"/>
@@ -4823,7 +5577,7 @@
         <v>0</v>
       </c>
       <c r="Q12" s="7">
-        <v>1.9E-2</v>
+        <v>0.02</v>
       </c>
       <c r="R12" s="15" t="str">
         <f t="shared" si="2"/>
@@ -4852,45 +5606,45 @@
         <v>1473</v>
       </c>
       <c r="E13" s="7">
-        <v>1468</v>
+        <v>1441</v>
       </c>
       <c r="F13" s="14">
         <f t="shared" si="0"/>
-        <v>3.3944331296673624E-3</v>
+        <v>2.1724372029870986E-2</v>
       </c>
       <c r="G13" s="7">
-        <v>0.14741199999999999</v>
+        <v>5.0251999999999998E-2</v>
       </c>
       <c r="H13" s="7">
-        <v>1.6620000000000001E-3</v>
+        <v>9.8700000000000003E-4</v>
       </c>
       <c r="I13" s="7">
-        <v>6.6140000000000001E-3</v>
+        <v>6.5009999999999998E-3</v>
       </c>
       <c r="J13" s="7">
-        <v>9.0790000000000003E-3</v>
+        <v>1.2090999999999999E-2</v>
       </c>
       <c r="K13" s="7">
-        <v>3.9199999999999999E-4</v>
+        <v>5.1500000000000005E-4</v>
       </c>
       <c r="L13" s="7">
         <v>3.2729999999999999E-3</v>
       </c>
       <c r="M13" s="15">
         <f t="shared" si="1"/>
-        <v>0.14741199999999999</v>
+        <v>5.0251999999999998E-2</v>
       </c>
       <c r="N13" s="7">
         <v>0</v>
       </c>
       <c r="O13" s="7">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="P13" s="7">
         <v>3</v>
       </c>
       <c r="Q13" s="7">
-        <v>8.5999999999999993E-2</v>
+        <v>0.09</v>
       </c>
       <c r="R13" s="15" t="str">
         <f t="shared" si="2"/>
@@ -4902,7 +5656,7 @@
       </c>
       <c r="T13" s="18">
         <f t="shared" si="3"/>
-        <v>11.388442521631644</v>
+        <v>3.8822620519159452</v>
       </c>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
@@ -4957,7 +5711,7 @@
         <v>0</v>
       </c>
       <c r="Q14" s="7">
-        <v>0.218</v>
+        <v>0.249</v>
       </c>
       <c r="R14" s="15" t="str">
         <f t="shared" si="2"/>
@@ -4986,45 +5740,45 @@
         <v>13790</v>
       </c>
       <c r="E15" s="7">
-        <v>5231</v>
+        <v>5136</v>
       </c>
       <c r="F15" s="14">
         <f t="shared" si="0"/>
-        <v>0.62066715010877449</v>
+        <v>0.62755620014503255</v>
       </c>
       <c r="G15" s="7">
-        <v>7.9950000000000004E-3</v>
+        <v>7.7270000000000004E-3</v>
       </c>
       <c r="H15" s="7">
-        <v>4.0499999999999998E-4</v>
+        <v>3.9399999999999998E-4</v>
       </c>
       <c r="I15" s="7">
-        <v>1.804E-3</v>
+        <v>1.818E-3</v>
       </c>
       <c r="J15" s="7">
-        <v>4.1469999999999996E-3</v>
+        <v>3.3059999999999999E-3</v>
       </c>
       <c r="K15" s="7">
-        <v>3.8999999999999999E-4</v>
+        <v>3.8699999999999997E-4</v>
       </c>
       <c r="L15" s="7">
-        <v>1.3600000000000001E-3</v>
+        <v>1.333E-3</v>
       </c>
       <c r="M15" s="15">
         <f t="shared" si="1"/>
-        <v>7.9950000000000004E-3</v>
+        <v>7.7270000000000004E-3</v>
       </c>
       <c r="N15" s="7">
         <v>0</v>
       </c>
       <c r="O15" s="7">
-        <v>865</v>
+        <v>817</v>
       </c>
       <c r="P15" s="7">
         <v>3</v>
       </c>
       <c r="Q15" s="7">
-        <v>0.81</v>
+        <v>1.042</v>
       </c>
       <c r="R15" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5036,7 +5790,7 @@
       </c>
       <c r="T15" s="18">
         <f t="shared" si="3"/>
-        <v>2.3980203959208164</v>
+        <v>2.317636472705459</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
@@ -5091,7 +5845,7 @@
         <v>0</v>
       </c>
       <c r="Q16" s="7">
-        <v>3.1E-2</v>
+        <v>3.5999999999999997E-2</v>
       </c>
       <c r="R16" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5158,7 +5912,7 @@
         <v>3</v>
       </c>
       <c r="Q17" s="7">
-        <v>0.112</v>
+        <v>0.14499999999999999</v>
       </c>
       <c r="R17" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5225,7 +5979,7 @@
         <v>0</v>
       </c>
       <c r="Q18" s="7">
-        <v>0.04</v>
+        <v>4.7E-2</v>
       </c>
       <c r="R18" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5254,26 +6008,26 @@
         <v>3410</v>
       </c>
       <c r="E19" s="7">
-        <v>1066</v>
+        <v>1014</v>
       </c>
       <c r="F19" s="14">
         <f t="shared" si="0"/>
-        <v>0.68739002932551319</v>
+        <v>0.70263929618768328</v>
       </c>
       <c r="G19" s="7">
         <v>6.2509999999999996E-3</v>
       </c>
       <c r="H19" s="7">
-        <v>6.3000000000000003E-4</v>
+        <v>6.5200000000000002E-4</v>
       </c>
       <c r="I19" s="7">
-        <v>2.7200000000000002E-3</v>
+        <v>2.8549999999999999E-3</v>
       </c>
       <c r="J19" s="7">
         <v>6.8649999999999996E-3</v>
       </c>
       <c r="K19" s="7">
-        <v>1.544E-3</v>
+        <v>1.5460000000000001E-3</v>
       </c>
       <c r="L19" s="7">
         <v>4.8919999999999996E-3</v>
@@ -5292,7 +6046,7 @@
         <v>2</v>
       </c>
       <c r="Q19" s="7">
-        <v>6.5000000000000002E-2</v>
+        <v>7.8E-2</v>
       </c>
       <c r="R19" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5359,7 +6113,7 @@
         <v>0</v>
       </c>
       <c r="Q20" s="7">
-        <v>3.6999999999999998E-2</v>
+        <v>4.3999999999999997E-2</v>
       </c>
       <c r="R20" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5388,45 +6142,45 @@
         <v>2926</v>
       </c>
       <c r="E21" s="7">
-        <v>2730</v>
+        <v>2189</v>
       </c>
       <c r="F21" s="14">
         <f t="shared" si="0"/>
-        <v>6.6985645933014371E-2</v>
+        <v>0.25187969924812026</v>
       </c>
       <c r="G21" s="7">
-        <v>1.3249E-2</v>
+        <v>9.7439999999999992E-3</v>
       </c>
       <c r="H21" s="7">
-        <v>3.3399999999999999E-4</v>
+        <v>2.03E-4</v>
       </c>
       <c r="I21" s="7">
-        <v>1.8649999999999999E-3</v>
+        <v>1.2409999999999999E-3</v>
       </c>
       <c r="J21" s="7">
-        <v>3.009E-3</v>
+        <v>4.1029999999999999E-3</v>
       </c>
       <c r="K21" s="7">
-        <v>1.3300000000000001E-4</v>
+        <v>2.2599999999999999E-4</v>
       </c>
       <c r="L21" s="7">
-        <v>8.3000000000000001E-4</v>
+        <v>1.1440000000000001E-3</v>
       </c>
       <c r="M21" s="15">
         <f t="shared" si="1"/>
-        <v>1.3249E-2</v>
+        <v>9.7439999999999992E-3</v>
       </c>
       <c r="N21" s="7">
         <v>0</v>
       </c>
       <c r="O21" s="7">
-        <v>861</v>
+        <v>702</v>
       </c>
       <c r="P21" s="7">
         <v>3</v>
       </c>
       <c r="Q21" s="7">
-        <v>0.129</v>
+        <v>0.14199999999999999</v>
       </c>
       <c r="R21" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5438,7 +6192,7 @@
       </c>
       <c r="T21" s="18">
         <f t="shared" si="3"/>
-        <v>4.992087415222306</v>
+        <v>3.6714393368500366</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.25">
@@ -5493,7 +6247,7 @@
         <v>0</v>
       </c>
       <c r="Q22" s="7">
-        <v>2.7069999999999999</v>
+        <v>3.226</v>
       </c>
       <c r="R22" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5522,45 +6276,45 @@
         <v>211874</v>
       </c>
       <c r="E23" s="7">
-        <v>42555</v>
+        <v>21172</v>
       </c>
       <c r="F23" s="14">
         <f t="shared" si="0"/>
-        <v>0.79914949451088857</v>
+        <v>0.90007268470883639</v>
       </c>
       <c r="G23" s="7">
-        <v>5.5662999999999997E-2</v>
+        <v>4.7434999999999998E-2</v>
       </c>
       <c r="H23" s="7">
-        <v>7.6000000000000004E-4</v>
+        <v>5.4799999999999998E-4</v>
       </c>
       <c r="I23" s="7">
-        <v>3.7959999999999999E-3</v>
+        <v>2.3040000000000001E-3</v>
       </c>
       <c r="J23" s="7">
-        <v>2.1922000000000001E-2</v>
+        <v>5.0117000000000002E-2</v>
       </c>
       <c r="K23" s="7">
-        <v>1.407E-3</v>
+        <v>3.483E-3</v>
       </c>
       <c r="L23" s="7">
-        <v>5.9709999999999997E-3</v>
+        <v>1.7822999999999999E-2</v>
       </c>
       <c r="M23" s="15">
         <f t="shared" si="1"/>
-        <v>5.5662999999999997E-2</v>
+        <v>5.0117000000000002E-2</v>
       </c>
       <c r="N23" s="7">
         <v>0</v>
       </c>
       <c r="O23" s="7">
-        <v>4149</v>
+        <v>0</v>
       </c>
       <c r="P23" s="7">
         <v>3</v>
       </c>
       <c r="Q23" s="7">
-        <v>9.923</v>
+        <v>12.196</v>
       </c>
       <c r="R23" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5572,7 +6326,7 @@
       </c>
       <c r="T23" s="18">
         <f t="shared" si="3"/>
-        <v>2.4262488013250807</v>
+        <v>2.184508761223956</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.25">
@@ -5627,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="Q24" s="7">
-        <v>5.7249999999999996</v>
+        <v>6.6929999999999996</v>
       </c>
       <c r="R24" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5656,45 +6410,45 @@
         <v>446670</v>
       </c>
       <c r="E25" s="7">
-        <v>150195</v>
+        <v>44633</v>
       </c>
       <c r="F25" s="14">
         <f t="shared" si="0"/>
-        <v>0.66374504667875611</v>
+        <v>0.9000761188349341</v>
       </c>
       <c r="G25" s="7">
-        <v>0.221384</v>
+        <v>2.4506E-2</v>
       </c>
       <c r="H25" s="7">
-        <v>1.9595999999999999E-2</v>
+        <v>3.7500000000000001E-4</v>
       </c>
       <c r="I25" s="7">
-        <v>0.15328600000000001</v>
+        <v>1.4350000000000001E-3</v>
       </c>
       <c r="J25" s="7">
-        <v>1.8332000000000001E-2</v>
+        <v>3.6756999999999998E-2</v>
       </c>
       <c r="K25" s="7">
-        <v>6.9999999999999999E-4</v>
+        <v>1.1379999999999999E-3</v>
       </c>
       <c r="L25" s="7">
-        <v>3.1199999999999999E-3</v>
+        <v>4.7889999999999999E-3</v>
       </c>
       <c r="M25" s="15">
         <f t="shared" si="1"/>
-        <v>0.221384</v>
+        <v>3.6756999999999998E-2</v>
       </c>
       <c r="N25" s="7">
         <v>0</v>
       </c>
       <c r="O25" s="7">
-        <v>15225</v>
+        <v>0</v>
       </c>
       <c r="P25" s="7">
         <v>3</v>
       </c>
       <c r="Q25" s="7">
-        <v>140.315</v>
+        <v>166.672</v>
       </c>
       <c r="R25" s="15" t="str">
         <f t="shared" si="2"/>
@@ -5706,7 +6460,7 @@
       </c>
       <c r="T25" s="18">
         <f t="shared" si="3"/>
-        <v>11.78828541001065</v>
+        <v>1.9572417465388712</v>
       </c>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.25">
@@ -5761,7 +6515,7 @@
         <v>0</v>
       </c>
       <c r="Q26">
-        <v>1.2390000000000001</v>
+        <v>1.274</v>
       </c>
       <c r="R26" t="str">
         <f t="shared" si="2"/>
@@ -5828,7 +6582,7 @@
         <v>1</v>
       </c>
       <c r="Q27">
-        <v>0.34499999999999997</v>
+        <v>0.40100000000000002</v>
       </c>
       <c r="R27" t="str">
         <f t="shared" si="2"/>
@@ -5895,7 +6649,7 @@
         <v>0</v>
       </c>
       <c r="Q28">
-        <v>8.0739999999999998</v>
+        <v>8.1780000000000008</v>
       </c>
       <c r="R28" t="str">
         <f t="shared" si="2"/>
@@ -5924,45 +6678,45 @@
         <v>405680</v>
       </c>
       <c r="E29">
-        <v>98032</v>
+        <v>40563</v>
       </c>
       <c r="F29">
         <f t="shared" si="0"/>
-        <v>0.75835140997830797</v>
+        <v>0.90001232498521</v>
       </c>
       <c r="G29">
-        <v>0.36501400000000001</v>
+        <v>2.0625000000000001E-2</v>
       </c>
       <c r="H29">
-        <v>1.3302E-2</v>
+        <v>9.8999999999999999E-4</v>
       </c>
       <c r="I29">
-        <v>0.108886</v>
+        <v>3.8470000000000002E-3</v>
       </c>
       <c r="J29">
-        <v>3.5890999999999999E-2</v>
+        <v>5.0375999999999997E-2</v>
       </c>
       <c r="K29">
-        <v>1.0380000000000001E-3</v>
+        <v>1.4059999999999999E-3</v>
       </c>
       <c r="L29">
-        <v>3.859E-3</v>
+        <v>4.999E-3</v>
       </c>
       <c r="M29">
         <f t="shared" si="1"/>
-        <v>0.36501400000000001</v>
+        <v>5.0375999999999997E-2</v>
       </c>
       <c r="N29">
         <v>0</v>
       </c>
       <c r="O29">
-        <v>4044</v>
+        <v>0</v>
       </c>
       <c r="P29">
         <v>3</v>
       </c>
       <c r="Q29">
-        <v>80.122</v>
+        <v>78.183000000000007</v>
       </c>
       <c r="R29" t="str">
         <f t="shared" si="2"/>
@@ -5974,7 +6728,7 @@
       </c>
       <c r="T29" s="20">
         <f t="shared" si="3"/>
-        <v>7.5022403091215519</v>
+        <v>1.0353927734615858</v>
       </c>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.25">
@@ -6029,7 +6783,7 @@
         <v>0</v>
       </c>
       <c r="Q30">
-        <v>6.0999999999999999E-2</v>
+        <v>5.3999999999999999E-2</v>
       </c>
       <c r="R30" t="str">
         <f t="shared" si="2"/>
@@ -6058,45 +6812,45 @@
         <v>5912</v>
       </c>
       <c r="E31">
-        <v>5129</v>
+        <v>4579</v>
       </c>
       <c r="F31">
         <f t="shared" si="0"/>
-        <v>0.13244248985115026</v>
+        <v>0.22547361299052771</v>
       </c>
       <c r="G31">
-        <v>8.3280000000000003E-3</v>
+        <v>8.0809999999999996E-3</v>
       </c>
       <c r="H31">
-        <v>2.72E-4</v>
+        <v>3.1500000000000001E-4</v>
       </c>
       <c r="I31">
-        <v>1.6739999999999999E-3</v>
+        <v>2.4260000000000002E-3</v>
       </c>
       <c r="J31">
-        <v>2.3149999999999998E-3</v>
+        <v>5.62E-3</v>
       </c>
       <c r="K31">
-        <v>2.6400000000000002E-4</v>
+        <v>4.55E-4</v>
       </c>
       <c r="L31">
-        <v>1.3339999999999999E-3</v>
+        <v>2.1299999999999999E-3</v>
       </c>
       <c r="M31">
         <f t="shared" si="1"/>
-        <v>8.3280000000000003E-3</v>
+        <v>8.0809999999999996E-3</v>
       </c>
       <c r="N31">
         <v>0</v>
       </c>
       <c r="O31">
-        <v>10386</v>
+        <v>9561</v>
       </c>
       <c r="P31">
         <v>3</v>
       </c>
       <c r="Q31">
-        <v>0.26700000000000002</v>
+        <v>0.27900000000000003</v>
       </c>
       <c r="R31" t="str">
         <f t="shared" si="2"/>
@@ -6108,7 +6862,7 @@
       </c>
       <c r="T31" s="20">
         <f t="shared" si="3"/>
-        <v>3.5788568972926518</v>
+        <v>3.4727116458960032</v>
       </c>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.25">
@@ -6163,7 +6917,7 @@
         <v>0</v>
       </c>
       <c r="Q32">
-        <v>0.18099999999999999</v>
+        <v>0.17899999999999999</v>
       </c>
       <c r="R32" t="str">
         <f t="shared" si="2"/>
@@ -6192,29 +6946,29 @@
         <v>16694</v>
       </c>
       <c r="E33">
-        <v>11921</v>
+        <v>11807</v>
       </c>
       <c r="F33">
         <f t="shared" si="0"/>
-        <v>0.28591110578651013</v>
+        <v>0.29273990655325266</v>
       </c>
       <c r="G33">
         <v>6.045E-3</v>
       </c>
       <c r="H33">
-        <v>1.11E-4</v>
+        <v>1.12E-4</v>
       </c>
       <c r="I33">
-        <v>5.9199999999999997E-4</v>
+        <v>6.0400000000000004E-4</v>
       </c>
       <c r="J33">
-        <v>3.0230000000000001E-3</v>
+        <v>4.8539999999999998E-3</v>
       </c>
       <c r="K33">
-        <v>3.0600000000000001E-4</v>
+        <v>3.1599999999999998E-4</v>
       </c>
       <c r="L33">
-        <v>1.4760000000000001E-3</v>
+        <v>1.5219999999999999E-3</v>
       </c>
       <c r="M33">
         <f t="shared" si="1"/>
@@ -6224,13 +6978,13 @@
         <v>0</v>
       </c>
       <c r="O33">
-        <v>24277</v>
+        <v>24206</v>
       </c>
       <c r="P33">
         <v>3</v>
       </c>
       <c r="Q33">
-        <v>0.70399999999999996</v>
+        <v>0.73599999999999999</v>
       </c>
       <c r="R33" t="str">
         <f t="shared" si="2"/>
@@ -6297,7 +7051,7 @@
         <v>0</v>
       </c>
       <c r="Q34">
-        <v>0.64600000000000002</v>
+        <v>0.63900000000000001</v>
       </c>
       <c r="R34" t="str">
         <f t="shared" si="2"/>
@@ -6364,7 +7118,7 @@
         <v>2</v>
       </c>
       <c r="Q35">
-        <v>0.81</v>
+        <v>0.84199999999999997</v>
       </c>
       <c r="R35" t="str">
         <f t="shared" si="2"/>
@@ -6431,7 +7185,7 @@
         <v>0</v>
       </c>
       <c r="Q36">
-        <v>0.48299999999999998</v>
+        <v>0.45600000000000002</v>
       </c>
       <c r="R36" t="str">
         <f t="shared" si="2"/>
@@ -6498,7 +7252,7 @@
         <v>1</v>
       </c>
       <c r="Q37">
-        <v>0.159</v>
+        <v>0.185</v>
       </c>
       <c r="R37" t="str">
         <f t="shared" si="2"/>
@@ -6565,7 +7319,7 @@
         <v>0</v>
       </c>
       <c r="Q38">
-        <v>3.863</v>
+        <v>3.7170000000000001</v>
       </c>
       <c r="R38" t="str">
         <f t="shared" si="2"/>
@@ -6632,7 +7386,7 @@
         <v>1</v>
       </c>
       <c r="Q39">
-        <v>1.4970000000000001</v>
+        <v>1.556</v>
       </c>
       <c r="R39" t="str">
         <f t="shared" si="2"/>
@@ -6699,7 +7453,7 @@
         <v>0</v>
       </c>
       <c r="Q40">
-        <v>25.439</v>
+        <v>24.951000000000001</v>
       </c>
       <c r="R40" t="str">
         <f t="shared" si="2"/>
@@ -6766,7 +7520,7 @@
         <v>1</v>
       </c>
       <c r="Q41">
-        <v>12.962</v>
+        <v>14.454000000000001</v>
       </c>
       <c r="R41" t="str">
         <f t="shared" si="2"/>
@@ -6833,7 +7587,7 @@
         <v>0</v>
       </c>
       <c r="Q42">
-        <v>0.35799999999999998</v>
+        <v>0.36599999999999999</v>
       </c>
       <c r="R42" t="str">
         <f t="shared" si="2"/>
@@ -6862,45 +7616,45 @@
         <v>31400</v>
       </c>
       <c r="E43">
-        <v>24908</v>
+        <v>22630</v>
       </c>
       <c r="F43">
         <f t="shared" si="0"/>
-        <v>0.20675159235668794</v>
+        <v>0.27929936305732483</v>
       </c>
       <c r="G43">
-        <v>0.151949</v>
+        <v>0.12346</v>
       </c>
       <c r="H43">
-        <v>2.496E-3</v>
+        <v>2.5530000000000001E-3</v>
       </c>
       <c r="I43">
-        <v>1.4452E-2</v>
+        <v>1.4726E-2</v>
       </c>
       <c r="J43">
-        <v>2.7682999999999999E-2</v>
+        <v>5.1305999999999997E-2</v>
       </c>
       <c r="K43">
-        <v>2.9610000000000001E-3</v>
+        <v>4.3949999999999996E-3</v>
       </c>
       <c r="L43">
-        <v>1.3044999999999999E-2</v>
+        <v>1.9809E-2</v>
       </c>
       <c r="M43">
         <f t="shared" si="1"/>
-        <v>0.151949</v>
+        <v>0.12346</v>
       </c>
       <c r="N43">
         <v>0</v>
       </c>
       <c r="O43">
-        <v>46048</v>
+        <v>42993</v>
       </c>
       <c r="P43">
         <v>3</v>
       </c>
       <c r="Q43">
-        <v>2.556</v>
+        <v>3.0070000000000001</v>
       </c>
       <c r="R43" t="str">
         <f t="shared" si="2"/>
@@ -6912,7 +7666,7 @@
       </c>
       <c r="T43" s="20">
         <f t="shared" si="3"/>
-        <v>6.1949200913242013</v>
+        <v>5.0334311806914549</v>
       </c>
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.25">
@@ -7452,26 +8206,26 @@
         <v>13790</v>
       </c>
       <c r="D6" s="7">
-        <v>9089</v>
+        <v>7155</v>
       </c>
       <c r="E6" s="14">
         <f t="shared" si="0"/>
-        <v>0.34089920232052207</v>
+        <v>0.48114575779550395</v>
       </c>
       <c r="F6" s="7">
         <v>3</v>
       </c>
       <c r="G6" s="7">
-        <v>2301</v>
+        <v>1747</v>
       </c>
       <c r="H6" s="7">
-        <v>1.7493000000000002E-2</v>
+        <v>1.1916E-2</v>
       </c>
       <c r="I6" s="7">
-        <v>2.3900000000000001E-4</v>
+        <v>2.8200000000000002E-4</v>
       </c>
       <c r="J6" s="7">
-        <v>9.3199999999999999E-4</v>
+        <v>1.14E-3</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -7485,26 +8239,26 @@
         <v>13790</v>
       </c>
       <c r="D7" s="7">
-        <v>5231</v>
+        <v>5136</v>
       </c>
       <c r="E7" s="14">
         <f t="shared" si="0"/>
-        <v>0.62066715010877449</v>
+        <v>0.62755620014503255</v>
       </c>
       <c r="F7" s="7">
         <v>3</v>
       </c>
       <c r="G7" s="7">
-        <v>865</v>
+        <v>817</v>
       </c>
       <c r="H7" s="7">
-        <v>7.9950000000000004E-3</v>
+        <v>7.7270000000000004E-3</v>
       </c>
       <c r="I7" s="7">
-        <v>3.9399999999999998E-4</v>
+        <v>3.8900000000000002E-4</v>
       </c>
       <c r="J7" s="7">
-        <v>1.4450000000000001E-3</v>
+        <v>1.4289999999999999E-3</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -7584,26 +8338,26 @@
         <v>211874</v>
       </c>
       <c r="D10" s="7">
-        <v>96954</v>
+        <v>21172</v>
       </c>
       <c r="E10" s="14">
         <f t="shared" si="0"/>
-        <v>0.54239784022579451</v>
+        <v>0.90007268470883639</v>
       </c>
       <c r="F10" s="7">
         <v>3</v>
       </c>
       <c r="G10" s="7">
-        <v>24710</v>
+        <v>0</v>
       </c>
       <c r="H10" s="7">
-        <v>0.19429399999999999</v>
+        <v>5.0117000000000002E-2</v>
       </c>
       <c r="I10" s="7">
-        <v>1.7030000000000001E-3</v>
+        <v>3.2160000000000001E-3</v>
       </c>
       <c r="J10" s="7">
-        <v>2.2160000000000001E-3</v>
+        <v>1.6778999999999999E-2</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -7617,26 +8371,26 @@
         <v>211874</v>
       </c>
       <c r="D11" s="7">
-        <v>66527</v>
+        <v>21172</v>
       </c>
       <c r="E11" s="14">
         <f t="shared" si="0"/>
-        <v>0.68600677761310969</v>
+        <v>0.90007268470883639</v>
       </c>
       <c r="F11" s="7">
         <v>3</v>
       </c>
       <c r="G11" s="7">
-        <v>12703</v>
+        <v>0</v>
       </c>
       <c r="H11" s="7">
-        <v>9.9413000000000001E-2</v>
+        <v>5.0117000000000002E-2</v>
       </c>
       <c r="I11" s="7">
-        <v>1.2149999999999999E-3</v>
+        <v>3.2160000000000001E-3</v>
       </c>
       <c r="J11" s="7">
-        <v>3.9370000000000004E-3</v>
+        <v>1.6778999999999999E-2</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -7650,26 +8404,26 @@
         <v>211874</v>
       </c>
       <c r="D12" s="7">
-        <v>42555</v>
+        <v>21172</v>
       </c>
       <c r="E12" s="14">
         <f t="shared" si="0"/>
-        <v>0.79914949451088857</v>
+        <v>0.90007268470883639</v>
       </c>
       <c r="F12" s="7">
         <v>3</v>
       </c>
       <c r="G12" s="7">
-        <v>4149</v>
+        <v>0</v>
       </c>
       <c r="H12" s="7">
-        <v>5.5662999999999997E-2</v>
+        <v>5.0117000000000002E-2</v>
       </c>
       <c r="I12" s="7">
-        <v>1.299E-3</v>
+        <v>3.2160000000000001E-3</v>
       </c>
       <c r="J12" s="7">
-        <v>5.7930000000000004E-3</v>
+        <v>1.6778999999999999E-2</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -7749,26 +8503,26 @@
         <v>405680</v>
       </c>
       <c r="D15" s="7">
-        <v>125308</v>
+        <v>40563</v>
       </c>
       <c r="E15" s="14">
         <f t="shared" si="0"/>
-        <v>0.69111615066061916</v>
+        <v>0.90001232498521</v>
       </c>
       <c r="F15" s="7">
         <v>3</v>
       </c>
       <c r="G15" s="7">
-        <v>9795</v>
+        <v>0</v>
       </c>
       <c r="H15" s="7">
-        <v>0.39617200000000002</v>
+        <v>5.0375999999999997E-2</v>
       </c>
       <c r="I15" s="7">
-        <v>3.6740000000000002E-3</v>
+        <v>1.3680000000000001E-3</v>
       </c>
       <c r="J15" s="7">
-        <v>4.6560000000000004E-3</v>
+        <v>4.9030000000000002E-3</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -7782,26 +8536,26 @@
         <v>405680</v>
       </c>
       <c r="D16" s="7">
-        <v>106515</v>
+        <v>40563</v>
       </c>
       <c r="E16" s="14">
         <f t="shared" si="0"/>
-        <v>0.73744084007099198</v>
+        <v>0.90001232498521</v>
       </c>
       <c r="F16" s="7">
         <v>3</v>
       </c>
       <c r="G16" s="7">
-        <v>5707</v>
+        <v>0</v>
       </c>
       <c r="H16" s="7">
-        <v>0.35922599999999999</v>
+        <v>5.0375999999999997E-2</v>
       </c>
       <c r="I16" s="7">
-        <v>3.2179999999999999E-3</v>
+        <v>1.3680000000000001E-3</v>
       </c>
       <c r="J16" s="7">
-        <v>4.9509999999999997E-3</v>
+        <v>4.9030000000000002E-3</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -7815,26 +8569,26 @@
         <v>405680</v>
       </c>
       <c r="D17" s="7">
-        <v>98032</v>
+        <v>40563</v>
       </c>
       <c r="E17" s="14">
         <f t="shared" si="0"/>
-        <v>0.75835140997830797</v>
+        <v>0.90001232498521</v>
       </c>
       <c r="F17" s="7">
         <v>3</v>
       </c>
       <c r="G17" s="7">
-        <v>4044</v>
+        <v>0</v>
       </c>
       <c r="H17" s="7">
-        <v>0.36501400000000001</v>
+        <v>5.0375999999999997E-2</v>
       </c>
       <c r="I17" s="7">
-        <v>3.4250000000000001E-3</v>
+        <v>1.3680000000000001E-3</v>
       </c>
       <c r="J17" s="7">
-        <v>5.2230000000000002E-3</v>
+        <v>4.9030000000000002E-3</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -8079,26 +8833,26 @@
         <v>1869988</v>
       </c>
       <c r="D25" s="7">
-        <v>575314</v>
+        <v>572915</v>
       </c>
       <c r="E25" s="14">
         <f t="shared" si="0"/>
-        <v>0.69234348027901782</v>
+        <v>0.69362637621203982</v>
       </c>
       <c r="F25" s="7">
         <v>3</v>
       </c>
       <c r="G25" s="7">
-        <v>191779</v>
+        <v>188994</v>
       </c>
       <c r="H25" s="7">
         <v>1.2324E-2</v>
       </c>
       <c r="I25" s="7">
-        <v>1.4779999999999999E-3</v>
+        <v>1.488E-3</v>
       </c>
       <c r="J25" s="7">
-        <v>4.0359999999999997E-3</v>
+        <v>4.058E-3</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -8407,24 +9161,24 @@
         <v>13790</v>
       </c>
       <c r="D8" s="7">
-        <v>5231</v>
+        <v>5136</v>
       </c>
       <c r="E8" s="14">
         <f t="shared" si="0"/>
-        <v>0.62066715010877449</v>
+        <v>0.62755620014503255</v>
       </c>
       <c r="F8" s="7">
-        <v>11261</v>
+        <v>11441</v>
       </c>
       <c r="G8" s="7">
-        <v>1126</v>
+        <v>1144</v>
       </c>
       <c r="H8" s="14">
         <f t="shared" si="1"/>
-        <v>0.90000888020602077</v>
+        <v>0.90000874049471202</v>
       </c>
       <c r="I8" s="7">
-        <v>7.9950000000000004E-3</v>
+        <v>7.7270000000000004E-3</v>
       </c>
       <c r="J8" s="7">
         <v>3</v>
@@ -8441,24 +9195,24 @@
         <v>13790</v>
       </c>
       <c r="D9" s="7">
-        <v>6358</v>
+        <v>687</v>
       </c>
       <c r="E9" s="14">
         <f t="shared" si="0"/>
-        <v>0.53894126178390134</v>
+        <v>0.9501812907904279</v>
       </c>
       <c r="F9" s="7">
-        <v>9834</v>
+        <v>13790</v>
       </c>
       <c r="G9" s="7">
-        <v>491</v>
+        <v>688</v>
       </c>
       <c r="H9" s="14">
         <f t="shared" si="1"/>
-        <v>0.95007118161480575</v>
+        <v>0.95010877447425668</v>
       </c>
       <c r="I9" s="7">
-        <v>2.3931999999999998E-2</v>
+        <v>2.0927000000000001E-2</v>
       </c>
       <c r="J9" s="7">
         <v>3</v>
@@ -8577,24 +9331,24 @@
         <v>211874</v>
       </c>
       <c r="D13" s="7">
-        <v>42555</v>
+        <v>21172</v>
       </c>
       <c r="E13" s="14">
         <f t="shared" si="0"/>
-        <v>0.79914949451088857</v>
+        <v>0.90007268470883639</v>
       </c>
       <c r="F13" s="7">
-        <v>202363</v>
+        <v>211874</v>
       </c>
       <c r="G13" s="7">
-        <v>20236</v>
+        <v>21187</v>
       </c>
       <c r="H13" s="14">
         <f t="shared" si="1"/>
-        <v>0.90000148248444622</v>
+        <v>0.90000188791451519</v>
       </c>
       <c r="I13" s="7">
-        <v>5.5662999999999997E-2</v>
+        <v>5.0117000000000002E-2</v>
       </c>
       <c r="J13" s="7">
         <v>3</v>
@@ -8611,24 +9365,24 @@
         <v>211874</v>
       </c>
       <c r="D14" s="7">
-        <v>36457</v>
+        <v>10580</v>
       </c>
       <c r="E14" s="14">
         <f t="shared" si="0"/>
-        <v>0.82793075129558136</v>
+        <v>0.9500646610721466</v>
       </c>
       <c r="F14" s="7">
-        <v>196329</v>
+        <v>211874</v>
       </c>
       <c r="G14" s="7">
-        <v>9815</v>
+        <v>10593</v>
       </c>
       <c r="H14" s="14">
         <f t="shared" si="1"/>
-        <v>0.95000738556199038</v>
+        <v>0.95000330385040166</v>
       </c>
       <c r="I14" s="7">
-        <v>0.19270200000000001</v>
+        <v>5.2992999999999998E-2</v>
       </c>
       <c r="J14" s="7">
         <v>3</v>
@@ -8747,24 +9501,24 @@
         <v>405680</v>
       </c>
       <c r="D18" s="7">
-        <v>98032</v>
+        <v>40563</v>
       </c>
       <c r="E18" s="14">
         <f t="shared" si="0"/>
-        <v>0.75835140997830797</v>
+        <v>0.90001232498521</v>
       </c>
       <c r="F18" s="7">
-        <v>390925</v>
+        <v>405680</v>
       </c>
       <c r="G18" s="7">
-        <v>39092</v>
+        <v>40568</v>
       </c>
       <c r="H18" s="14">
         <f t="shared" si="1"/>
-        <v>0.90000127901771443</v>
+        <v>0.9</v>
       </c>
       <c r="I18" s="7">
-        <v>0.36501400000000001</v>
+        <v>5.0375999999999997E-2</v>
       </c>
       <c r="J18" s="7">
         <v>3</v>
@@ -8781,24 +9535,24 @@
         <v>405680</v>
       </c>
       <c r="D19" s="7">
-        <v>48046</v>
+        <v>20279</v>
       </c>
       <c r="E19" s="14">
         <f t="shared" si="0"/>
-        <v>0.88156675211989743</v>
+        <v>0.95001232498521004</v>
       </c>
       <c r="F19" s="7">
-        <v>401031</v>
+        <v>405680</v>
       </c>
       <c r="G19" s="7">
-        <v>20051</v>
+        <v>20284</v>
       </c>
       <c r="H19" s="14">
         <f t="shared" si="1"/>
-        <v>0.95000137146504882</v>
+        <v>0.95</v>
       </c>
       <c r="I19" s="7">
-        <v>0.31517000000000001</v>
+        <v>0.19516600000000001</v>
       </c>
       <c r="J19" s="7">
         <v>3</v>
@@ -9241,7 +9995,7 @@
         <v>0.16586300000000001</v>
       </c>
       <c r="I5" s="7">
-        <v>0.377</v>
+        <v>0.375</v>
       </c>
       <c r="J5" s="7">
         <v>0</v>
@@ -9280,7 +10034,7 @@
         <v>0.17016200000000001</v>
       </c>
       <c r="I6" s="7">
-        <v>0.621</v>
+        <v>0.59699999999999998</v>
       </c>
       <c r="J6" s="7">
         <v>0</v>
@@ -9358,7 +10112,7 @@
         <v>1.3436E-2</v>
       </c>
       <c r="I8" s="7">
-        <v>0.124</v>
+        <v>0.122</v>
       </c>
       <c r="J8" s="7">
         <v>0</v>
@@ -9397,7 +10151,7 @@
         <v>6.0574999999999997E-2</v>
       </c>
       <c r="I9" s="7">
-        <v>0.76900000000000002</v>
+        <v>0.77800000000000002</v>
       </c>
       <c r="J9" s="7">
         <v>0</v>
@@ -9436,7 +10190,7 @@
         <v>4.011E-2</v>
       </c>
       <c r="I10" s="7">
-        <v>1.3089999999999999</v>
+        <v>1.3859999999999999</v>
       </c>
       <c r="J10" s="7">
         <v>0</v>
@@ -9475,7 +10229,7 @@
         <v>6.3699999999999998E-4</v>
       </c>
       <c r="I11" s="7">
-        <v>0.01</v>
+        <v>1.0999999999999999E-2</v>
       </c>
       <c r="J11" s="7">
         <v>0</v>
@@ -9553,7 +10307,7 @@
         <v>8.2999999999999998E-5</v>
       </c>
       <c r="I13" s="7">
-        <v>0.112</v>
+        <v>0.11899999999999999</v>
       </c>
       <c r="J13" s="7">
         <v>0</v>
@@ -9592,7 +10346,7 @@
         <v>1.0610000000000001E-3</v>
       </c>
       <c r="I14" s="7">
-        <v>0.185</v>
+        <v>0.24199999999999999</v>
       </c>
       <c r="J14" s="7">
         <v>0</v>
@@ -9670,7 +10424,7 @@
         <v>1.5659999999999999E-3</v>
       </c>
       <c r="I16" s="7">
-        <v>3.3000000000000002E-2</v>
+        <v>3.1E-2</v>
       </c>
       <c r="J16" s="7">
         <v>0</v>
@@ -9709,7 +10463,7 @@
         <v>7.2999999999999999E-5</v>
       </c>
       <c r="I17" s="7">
-        <v>2.1999999999999999E-2</v>
+        <v>2.3E-2</v>
       </c>
       <c r="J17" s="7">
         <v>0</v>
@@ -9787,7 +10541,7 @@
         <v>1.2999999999999999E-4</v>
       </c>
       <c r="I19" s="7">
-        <v>1.7999999999999999E-2</v>
+        <v>1.9E-2</v>
       </c>
       <c r="J19" s="7">
         <v>0</v>
@@ -9826,7 +10580,7 @@
         <v>1.725E-3</v>
       </c>
       <c r="I20" s="7">
-        <v>3.3000000000000002E-2</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="J20" s="7">
         <v>0</v>
@@ -9904,7 +10658,7 @@
         <v>3.2160000000000001E-3</v>
       </c>
       <c r="I22" s="7">
-        <v>2.6480000000000001</v>
+        <v>2.5289999999999999</v>
       </c>
       <c r="J22" s="7">
         <v>0</v>
@@ -9943,7 +10697,7 @@
         <v>2.92E-4</v>
       </c>
       <c r="I23" s="7">
-        <v>3.206</v>
+        <v>3.15</v>
       </c>
       <c r="J23" s="7">
         <v>0</v>
@@ -9982,7 +10736,7 @@
         <v>1.0690000000000001E-3</v>
       </c>
       <c r="I24" s="7">
-        <v>5.4210000000000003</v>
+        <v>5.4329999999999998</v>
       </c>
       <c r="J24" s="7">
         <v>0</v>
@@ -10021,7 +10775,7 @@
         <v>1.3730000000000001E-3</v>
       </c>
       <c r="I25" s="7">
-        <v>0.76100000000000001</v>
+        <v>0.73399999999999999</v>
       </c>
       <c r="J25" s="7">
         <v>0</v>
@@ -10060,7 +10814,7 @@
         <v>3.8200000000000002E-4</v>
       </c>
       <c r="I26" s="7">
-        <v>1.2549999999999999</v>
+        <v>1.304</v>
       </c>
       <c r="J26" s="7">
         <v>0</v>
@@ -10099,7 +10853,7 @@
         <v>3.3599999999999998E-4</v>
       </c>
       <c r="I27" s="7">
-        <v>3.6179999999999999</v>
+        <v>3.6419999999999999</v>
       </c>
       <c r="J27" s="7">
         <v>0</v>
@@ -10138,7 +10892,7 @@
         <v>1.3680000000000001E-3</v>
       </c>
       <c r="I28" s="7">
-        <v>7.0069999999999997</v>
+        <v>8.17</v>
       </c>
       <c r="J28" s="7">
         <v>0</v>
@@ -10177,7 +10931,7 @@
         <v>1.6799999999999999E-4</v>
       </c>
       <c r="I29" s="7">
-        <v>4.2000000000000003E-2</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="J29" s="7">
         <v>0</v>
@@ -10216,7 +10970,7 @@
         <v>3.2160000000000001E-3</v>
       </c>
       <c r="I30" s="7">
-        <v>5.7000000000000002E-2</v>
+        <v>5.8000000000000003E-2</v>
       </c>
       <c r="J30" s="7">
         <v>0</v>
@@ -10255,7 +11009,7 @@
         <v>5.3000000000000001E-5</v>
       </c>
       <c r="I31" s="7">
-        <v>0.126</v>
+        <v>0.128</v>
       </c>
       <c r="J31" s="7">
         <v>0</v>
@@ -10294,7 +11048,7 @@
         <v>3.7810000000000001E-3</v>
       </c>
       <c r="I32" s="7">
-        <v>0.186</v>
+        <v>0.188</v>
       </c>
       <c r="J32" s="7">
         <v>0</v>
@@ -10333,7 +11087,7 @@
         <v>2.2000000000000001E-4</v>
       </c>
       <c r="I33" s="7">
-        <v>0.4</v>
+        <v>0.39600000000000002</v>
       </c>
       <c r="J33" s="7">
         <v>0</v>
@@ -10372,7 +11126,7 @@
         <v>5.2400000000000005E-4</v>
       </c>
       <c r="I34" s="7">
-        <v>0.66500000000000004</v>
+        <v>0.65400000000000003</v>
       </c>
       <c r="J34" s="7">
         <v>0</v>
@@ -10411,7 +11165,7 @@
         <v>2.24E-4</v>
       </c>
       <c r="I35" s="7">
-        <v>0.36499999999999999</v>
+        <v>0.36599999999999999</v>
       </c>
       <c r="J35" s="7">
         <v>0</v>
@@ -10450,7 +11204,7 @@
         <v>4.8000000000000001E-5</v>
       </c>
       <c r="I36" s="7">
-        <v>0.47299999999999998</v>
+        <v>0.48799999999999999</v>
       </c>
       <c r="J36" s="7">
         <v>0</v>
@@ -10489,7 +11243,7 @@
         <v>6.3159000000000007E-2</v>
       </c>
       <c r="I37" s="7">
-        <v>2.8519999999999999</v>
+        <v>2.7970000000000002</v>
       </c>
       <c r="J37" s="7">
         <v>0</v>
@@ -10528,7 +11282,7 @@
         <v>1.941E-2</v>
       </c>
       <c r="I38" s="7">
-        <v>3.8450000000000002</v>
+        <v>3.831</v>
       </c>
       <c r="J38" s="7">
         <v>0</v>
@@ -10567,7 +11321,7 @@
         <v>3.1000000000000001E-5</v>
       </c>
       <c r="I39" s="7">
-        <v>27.135000000000002</v>
+        <v>29.588000000000001</v>
       </c>
       <c r="J39" s="7">
         <v>0</v>
@@ -10606,7 +11360,7 @@
         <v>2.1870000000000001E-3</v>
       </c>
       <c r="I40" s="7">
-        <v>24.113</v>
+        <v>24.888999999999999</v>
       </c>
       <c r="J40" s="7">
         <v>0</v>
@@ -10645,7 +11399,7 @@
         <v>1.694E-3</v>
       </c>
       <c r="I41" s="7">
-        <v>0.29499999999999998</v>
+        <v>0.29299999999999998</v>
       </c>
       <c r="J41" s="7">
         <v>0</v>
@@ -10684,7 +11438,7 @@
         <v>2.3363999999999999E-2</v>
       </c>
       <c r="I42" s="7">
-        <v>0.35199999999999998</v>
+        <v>0.35</v>
       </c>
       <c r="J42" s="7">
         <v>0</v>

</xml_diff>